<commit_message>
results cal with tax at 250
</commit_message>
<xml_diff>
--- a/dataCaseStudy_WtE/raw_results/CaL/Summary.xlsx
+++ b/dataCaseStudy_WtE/raw_results/CaL/Summary.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE7"/>
+  <dimension ref="A1:AE13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1200,6 +1200,624 @@
       <c r="AE7" t="inlineStr">
         <is>
           <t>dataCaseStudy_WtE\raw_results\CaL\20260128113813_el_price_175_costs</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>60658269.93059336</v>
+      </c>
+      <c r="B8" t="n">
+        <v>7082943.251772646</v>
+      </c>
+      <c r="C8" t="n">
+        <v>0</v>
+      </c>
+      <c r="D8" t="n">
+        <v>5678990.357307213</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" t="n">
+        <v>12761933.60907986</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" t="n">
+        <v>116.2909854684303</v>
+      </c>
+      <c r="I8" t="n">
+        <v>-5359875.275964417</v>
+      </c>
+      <c r="J8" t="n">
+        <v>0</v>
+      </c>
+      <c r="K8" t="n">
+        <v>0</v>
+      </c>
+      <c r="L8" t="n">
+        <v>53256095.30649245</v>
+      </c>
+      <c r="M8" t="n">
+        <v>60658269.93059336</v>
+      </c>
+      <c r="N8" t="n">
+        <v>213024.3812259698</v>
+      </c>
+      <c r="O8" t="n">
+        <v>0</v>
+      </c>
+      <c r="P8" t="n">
+        <v>213024.3812259698</v>
+      </c>
+      <c r="Q8" t="n">
+        <v>213024.3812259698</v>
+      </c>
+      <c r="R8" t="n">
+        <v>0</v>
+      </c>
+      <c r="S8" t="n">
+        <v>0</v>
+      </c>
+      <c r="T8" t="n">
+        <v>0</v>
+      </c>
+      <c r="U8" t="n">
+        <v>0</v>
+      </c>
+      <c r="V8" t="n">
+        <v>3.024999856948853</v>
+      </c>
+      <c r="W8" t="n">
+        <v>60658269.93059336</v>
+      </c>
+      <c r="X8" t="n">
+        <v>60658269.93059336</v>
+      </c>
+      <c r="Y8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z8" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA8" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC8" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD8" t="inlineStr">
+        <is>
+          <t>el_price_50_costs</t>
+        </is>
+      </c>
+      <c r="AE8" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_WtE\raw_results\CaL\20260128134948_el_price_50_costs</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>56705650.20608237</v>
+      </c>
+      <c r="B9" t="n">
+        <v>23602309.58151861</v>
+      </c>
+      <c r="C9" t="n">
+        <v>3675691.270406743</v>
+      </c>
+      <c r="D9" t="n">
+        <v>17966626.69030973</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" t="n">
+        <v>41568936.27182833</v>
+      </c>
+      <c r="G9" t="n">
+        <v>3675691.270406743</v>
+      </c>
+      <c r="H9" t="n">
+        <v>1846706.630736768</v>
+      </c>
+      <c r="I9" t="n">
+        <v>-12877164.53350351</v>
+      </c>
+      <c r="J9" t="n">
+        <v>0</v>
+      </c>
+      <c r="K9" t="n">
+        <v>0</v>
+      </c>
+      <c r="L9" t="n">
+        <v>22491480.56661404</v>
+      </c>
+      <c r="M9" t="n">
+        <v>56705650.20608237</v>
+      </c>
+      <c r="N9" t="n">
+        <v>89969.36363936203</v>
+      </c>
+      <c r="O9" t="n">
+        <v>0</v>
+      </c>
+      <c r="P9" t="n">
+        <v>89969.36363936203</v>
+      </c>
+      <c r="Q9" t="n">
+        <v>89965.92226645617</v>
+      </c>
+      <c r="R9" t="n">
+        <v>0</v>
+      </c>
+      <c r="S9" t="n">
+        <v>0</v>
+      </c>
+      <c r="T9" t="n">
+        <v>0</v>
+      </c>
+      <c r="U9" t="n">
+        <v>3.441372905900046</v>
+      </c>
+      <c r="V9" t="n">
+        <v>2.953000068664551</v>
+      </c>
+      <c r="W9" t="n">
+        <v>56705650.20608237</v>
+      </c>
+      <c r="X9" t="n">
+        <v>56705650.20608237</v>
+      </c>
+      <c r="Y9" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z9" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA9" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC9" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD9" t="inlineStr">
+        <is>
+          <t>el_price_75_costs</t>
+        </is>
+      </c>
+      <c r="AE9" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_WtE\raw_results\CaL\20260128135205_el_price_75_costs</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>52229355.33047114</v>
+      </c>
+      <c r="B10" t="n">
+        <v>28580992.5973305</v>
+      </c>
+      <c r="C10" t="n">
+        <v>4148774.160734102</v>
+      </c>
+      <c r="D10" t="n">
+        <v>21569232.87215166</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" t="n">
+        <v>50150225.46948216</v>
+      </c>
+      <c r="G10" t="n">
+        <v>4148774.160734102</v>
+      </c>
+      <c r="H10" t="n">
+        <v>2330063.610840216</v>
+      </c>
+      <c r="I10" t="n">
+        <v>-18838351.33481684</v>
+      </c>
+      <c r="J10" t="n">
+        <v>0</v>
+      </c>
+      <c r="K10" t="n">
+        <v>0</v>
+      </c>
+      <c r="L10" t="n">
+        <v>14438643.42423149</v>
+      </c>
+      <c r="M10" t="n">
+        <v>52229355.33047114</v>
+      </c>
+      <c r="N10" t="n">
+        <v>57758.91587147661</v>
+      </c>
+      <c r="O10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P10" t="n">
+        <v>57758.91587147661</v>
+      </c>
+      <c r="Q10" t="n">
+        <v>57754.57369692596</v>
+      </c>
+      <c r="R10" t="n">
+        <v>0</v>
+      </c>
+      <c r="S10" t="n">
+        <v>0</v>
+      </c>
+      <c r="T10" t="n">
+        <v>0</v>
+      </c>
+      <c r="U10" t="n">
+        <v>4.34217455063829</v>
+      </c>
+      <c r="V10" t="n">
+        <v>2.885999917984009</v>
+      </c>
+      <c r="W10" t="n">
+        <v>52229355.33047114</v>
+      </c>
+      <c r="X10" t="n">
+        <v>52229355.33047114</v>
+      </c>
+      <c r="Y10" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z10" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA10" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC10" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD10" t="inlineStr">
+        <is>
+          <t>el_price_100_costs</t>
+        </is>
+      </c>
+      <c r="AE10" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_WtE\raw_results\CaL\20260128135426_el_price_100_costs</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>47434341.81768903</v>
+      </c>
+      <c r="B11" t="n">
+        <v>30170466.41311156</v>
+      </c>
+      <c r="C11" t="n">
+        <v>4299808.654089317</v>
+      </c>
+      <c r="D11" t="n">
+        <v>22711260.94737182</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" t="n">
+        <v>52881727.36048338</v>
+      </c>
+      <c r="G11" t="n">
+        <v>4299808.654089317</v>
+      </c>
+      <c r="H11" t="n">
+        <v>2488561.166745042</v>
+      </c>
+      <c r="I11" t="n">
+        <v>-24217404.64018829</v>
+      </c>
+      <c r="J11" t="n">
+        <v>0</v>
+      </c>
+      <c r="K11" t="n">
+        <v>0</v>
+      </c>
+      <c r="L11" t="n">
+        <v>11981649.27655958</v>
+      </c>
+      <c r="M11" t="n">
+        <v>47434341.81768903</v>
+      </c>
+      <c r="N11" t="n">
+        <v>47931.21586321186</v>
+      </c>
+      <c r="O11" t="n">
+        <v>0</v>
+      </c>
+      <c r="P11" t="n">
+        <v>47931.21586321186</v>
+      </c>
+      <c r="Q11" t="n">
+        <v>47926.59710623833</v>
+      </c>
+      <c r="R11" t="n">
+        <v>0</v>
+      </c>
+      <c r="S11" t="n">
+        <v>0</v>
+      </c>
+      <c r="T11" t="n">
+        <v>0</v>
+      </c>
+      <c r="U11" t="n">
+        <v>4.618756973548098</v>
+      </c>
+      <c r="V11" t="n">
+        <v>2.953999996185303</v>
+      </c>
+      <c r="W11" t="n">
+        <v>47434341.81768903</v>
+      </c>
+      <c r="X11" t="n">
+        <v>47434341.81768903</v>
+      </c>
+      <c r="Y11" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z11" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA11" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC11" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD11" t="inlineStr">
+        <is>
+          <t>el_price_125_costs</t>
+        </is>
+      </c>
+      <c r="AE11" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_WtE\raw_results\CaL\20260128135651_el_price_125_costs</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>42569275.14786529</v>
+      </c>
+      <c r="B12" t="n">
+        <v>30620008.39546236</v>
+      </c>
+      <c r="C12" t="n">
+        <v>4342524.894440144</v>
+      </c>
+      <c r="D12" t="n">
+        <v>23031257.4414313</v>
+      </c>
+      <c r="E12" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" t="n">
+        <v>53651265.83689366</v>
+      </c>
+      <c r="G12" t="n">
+        <v>4342524.894440144</v>
+      </c>
+      <c r="H12" t="n">
+        <v>2543368.416960416</v>
+      </c>
+      <c r="I12" t="n">
+        <v>-29309662.41969334</v>
+      </c>
+      <c r="J12" t="n">
+        <v>0</v>
+      </c>
+      <c r="K12" t="n">
+        <v>0</v>
+      </c>
+      <c r="L12" t="n">
+        <v>11341778.4192644</v>
+      </c>
+      <c r="M12" t="n">
+        <v>42569275.14786529</v>
+      </c>
+      <c r="N12" t="n">
+        <v>45371.80659959024</v>
+      </c>
+      <c r="O12" t="n">
+        <v>0</v>
+      </c>
+      <c r="P12" t="n">
+        <v>45371.80659959024</v>
+      </c>
+      <c r="Q12" t="n">
+        <v>45367.11367705761</v>
+      </c>
+      <c r="R12" t="n">
+        <v>0</v>
+      </c>
+      <c r="S12" t="n">
+        <v>0</v>
+      </c>
+      <c r="T12" t="n">
+        <v>0</v>
+      </c>
+      <c r="U12" t="n">
+        <v>4.692922532634418</v>
+      </c>
+      <c r="V12" t="n">
+        <v>3.101999998092651</v>
+      </c>
+      <c r="W12" t="n">
+        <v>42569275.14786529</v>
+      </c>
+      <c r="X12" t="n">
+        <v>42569275.14786529</v>
+      </c>
+      <c r="Y12" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z12" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA12" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB12" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC12" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD12" t="inlineStr">
+        <is>
+          <t>el_price_150_costs</t>
+        </is>
+      </c>
+      <c r="AE12" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_WtE\raw_results\CaL\20260128135910_el_price_150_costs</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>37663103.6152001</v>
+      </c>
+      <c r="B13" t="n">
+        <v>30920004.27095176</v>
+      </c>
+      <c r="C13" t="n">
+        <v>4371031.010497759</v>
+      </c>
+      <c r="D13" t="n">
+        <v>23243173.15400708</v>
+      </c>
+      <c r="E13" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" t="n">
+        <v>54163177.42495884</v>
+      </c>
+      <c r="G13" t="n">
+        <v>4371031.010497759</v>
+      </c>
+      <c r="H13" t="n">
+        <v>2633349.881300342</v>
+      </c>
+      <c r="I13" t="n">
+        <v>-34523115.31161098</v>
+      </c>
+      <c r="J13" t="n">
+        <v>0</v>
+      </c>
+      <c r="K13" t="n">
+        <v>0</v>
+      </c>
+      <c r="L13" t="n">
+        <v>11018660.61005414</v>
+      </c>
+      <c r="M13" t="n">
+        <v>37663103.6152001</v>
+      </c>
+      <c r="N13" t="n">
+        <v>44079.38264905868</v>
+      </c>
+      <c r="O13" t="n">
+        <v>0</v>
+      </c>
+      <c r="P13" t="n">
+        <v>44079.38264905868</v>
+      </c>
+      <c r="Q13" t="n">
+        <v>44074.64244021656</v>
+      </c>
+      <c r="R13" t="n">
+        <v>0</v>
+      </c>
+      <c r="S13" t="n">
+        <v>0</v>
+      </c>
+      <c r="T13" t="n">
+        <v>0</v>
+      </c>
+      <c r="U13" t="n">
+        <v>4.740208842091318</v>
+      </c>
+      <c r="V13" t="n">
+        <v>3.266000032424927</v>
+      </c>
+      <c r="W13" t="n">
+        <v>37663103.6152001</v>
+      </c>
+      <c r="X13" t="n">
+        <v>37663103.6152001</v>
+      </c>
+      <c r="Y13" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z13" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA13" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB13" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC13" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD13" t="inlineStr">
+        <is>
+          <t>el_price_175_costs</t>
+        </is>
+      </c>
+      <c r="AE13" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_WtE\raw_results\CaL\20260128140134_el_price_175_costs</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Rerun all wte results with correct gas price
</commit_message>
<xml_diff>
--- a/dataCaseStudy_WtE/raw_results/CaL/Summary.xlsx
+++ b/dataCaseStudy_WtE/raw_results/CaL/Summary.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE13"/>
+  <dimension ref="A1:AE23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1818,6 +1818,1036 @@
       <c r="AE13" t="inlineStr">
         <is>
           <t>dataCaseStudy_WtE\raw_results\CaL\20260128140134_el_price_175_costs</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>56705688.96974421</v>
+      </c>
+      <c r="B14" t="n">
+        <v>23602309.58151861</v>
+      </c>
+      <c r="C14" t="n">
+        <v>3675691.270406743</v>
+      </c>
+      <c r="D14" t="n">
+        <v>17966626.69030973</v>
+      </c>
+      <c r="E14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" t="n">
+        <v>41568936.27182833</v>
+      </c>
+      <c r="G14" t="n">
+        <v>3675691.270406743</v>
+      </c>
+      <c r="H14" t="n">
+        <v>1846745.394398591</v>
+      </c>
+      <c r="I14" t="n">
+        <v>-12877164.53350351</v>
+      </c>
+      <c r="J14" t="n">
+        <v>0</v>
+      </c>
+      <c r="K14" t="n">
+        <v>0</v>
+      </c>
+      <c r="L14" t="n">
+        <v>22491480.56661404</v>
+      </c>
+      <c r="M14" t="n">
+        <v>56705688.96974421</v>
+      </c>
+      <c r="N14" t="n">
+        <v>89969.36363936203</v>
+      </c>
+      <c r="O14" t="n">
+        <v>0</v>
+      </c>
+      <c r="P14" t="n">
+        <v>89969.36363936203</v>
+      </c>
+      <c r="Q14" t="n">
+        <v>89965.92226645617</v>
+      </c>
+      <c r="R14" t="n">
+        <v>0</v>
+      </c>
+      <c r="S14" t="n">
+        <v>0</v>
+      </c>
+      <c r="T14" t="n">
+        <v>0</v>
+      </c>
+      <c r="U14" t="n">
+        <v>3.441372905900046</v>
+      </c>
+      <c r="V14" t="n">
+        <v>3.20799994468689</v>
+      </c>
+      <c r="W14" t="n">
+        <v>56705688.96974421</v>
+      </c>
+      <c r="X14" t="n">
+        <v>56705688.96974421</v>
+      </c>
+      <c r="Y14" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z14" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA14" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC14" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD14" t="inlineStr">
+        <is>
+          <t>el_price_75_costs</t>
+        </is>
+      </c>
+      <c r="AE14" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_WtE\raw_results\CaL\20260128143522_el_price_75_costs</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>52229394.09413296</v>
+      </c>
+      <c r="B15" t="n">
+        <v>28580992.5973305</v>
+      </c>
+      <c r="C15" t="n">
+        <v>4148774.160734102</v>
+      </c>
+      <c r="D15" t="n">
+        <v>21569232.87215166</v>
+      </c>
+      <c r="E15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" t="n">
+        <v>50150225.46948216</v>
+      </c>
+      <c r="G15" t="n">
+        <v>4148774.160734102</v>
+      </c>
+      <c r="H15" t="n">
+        <v>2330102.374502039</v>
+      </c>
+      <c r="I15" t="n">
+        <v>-18838351.33481684</v>
+      </c>
+      <c r="J15" t="n">
+        <v>0</v>
+      </c>
+      <c r="K15" t="n">
+        <v>0</v>
+      </c>
+      <c r="L15" t="n">
+        <v>14438643.42423149</v>
+      </c>
+      <c r="M15" t="n">
+        <v>52229394.09413296</v>
+      </c>
+      <c r="N15" t="n">
+        <v>57758.91587147661</v>
+      </c>
+      <c r="O15" t="n">
+        <v>0</v>
+      </c>
+      <c r="P15" t="n">
+        <v>57758.91587147661</v>
+      </c>
+      <c r="Q15" t="n">
+        <v>57754.57369692596</v>
+      </c>
+      <c r="R15" t="n">
+        <v>0</v>
+      </c>
+      <c r="S15" t="n">
+        <v>0</v>
+      </c>
+      <c r="T15" t="n">
+        <v>0</v>
+      </c>
+      <c r="U15" t="n">
+        <v>4.34217455063829</v>
+      </c>
+      <c r="V15" t="n">
+        <v>2.991999864578247</v>
+      </c>
+      <c r="W15" t="n">
+        <v>52229394.09413296</v>
+      </c>
+      <c r="X15" t="n">
+        <v>52229394.09413296</v>
+      </c>
+      <c r="Y15" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z15" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA15" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC15" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD15" t="inlineStr">
+        <is>
+          <t>el_price_100_costs</t>
+        </is>
+      </c>
+      <c r="AE15" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_WtE\raw_results\CaL\20260128143742_el_price_100_costs</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>47436854.16685127</v>
+      </c>
+      <c r="B16" t="n">
+        <v>30170466.41311156</v>
+      </c>
+      <c r="C16" t="n">
+        <v>4299808.654089317</v>
+      </c>
+      <c r="D16" t="n">
+        <v>22711260.94737182</v>
+      </c>
+      <c r="E16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" t="n">
+        <v>52881727.36048338</v>
+      </c>
+      <c r="G16" t="n">
+        <v>4299808.654089317</v>
+      </c>
+      <c r="H16" t="n">
+        <v>2483596.055394794</v>
+      </c>
+      <c r="I16" t="n">
+        <v>-24200253.56808047</v>
+      </c>
+      <c r="J16" t="n">
+        <v>0</v>
+      </c>
+      <c r="K16" t="n">
+        <v>0</v>
+      </c>
+      <c r="L16" t="n">
+        <v>11971975.66496425</v>
+      </c>
+      <c r="M16" t="n">
+        <v>47436854.16685127</v>
+      </c>
+      <c r="N16" t="n">
+        <v>47892.52141683055</v>
+      </c>
+      <c r="O16" t="n">
+        <v>0</v>
+      </c>
+      <c r="P16" t="n">
+        <v>47892.52141683055</v>
+      </c>
+      <c r="Q16" t="n">
+        <v>47887.90265985703</v>
+      </c>
+      <c r="R16" t="n">
+        <v>0</v>
+      </c>
+      <c r="S16" t="n">
+        <v>0</v>
+      </c>
+      <c r="T16" t="n">
+        <v>0</v>
+      </c>
+      <c r="U16" t="n">
+        <v>4.618756973548098</v>
+      </c>
+      <c r="V16" t="n">
+        <v>2.953000068664551</v>
+      </c>
+      <c r="W16" t="n">
+        <v>47436854.16685127</v>
+      </c>
+      <c r="X16" t="n">
+        <v>47436854.16685127</v>
+      </c>
+      <c r="Y16" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z16" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA16" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC16" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD16" t="inlineStr">
+        <is>
+          <t>el_price_125_costs</t>
+        </is>
+      </c>
+      <c r="AE16" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_WtE\raw_results\CaL\20260128144005_el_price_125_costs</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>42575562.54061422</v>
+      </c>
+      <c r="B17" t="n">
+        <v>30620008.39546236</v>
+      </c>
+      <c r="C17" t="n">
+        <v>4342524.894440144</v>
+      </c>
+      <c r="D17" t="n">
+        <v>23031257.4414313</v>
+      </c>
+      <c r="E17" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" t="n">
+        <v>53651265.83689366</v>
+      </c>
+      <c r="G17" t="n">
+        <v>4342524.894440144</v>
+      </c>
+      <c r="H17" t="n">
+        <v>2535175.660100587</v>
+      </c>
+      <c r="I17" t="n">
+        <v>-29275991.16656995</v>
+      </c>
+      <c r="J17" t="n">
+        <v>0</v>
+      </c>
+      <c r="K17" t="n">
+        <v>0</v>
+      </c>
+      <c r="L17" t="n">
+        <v>11322587.31574978</v>
+      </c>
+      <c r="M17" t="n">
+        <v>42575562.54061422</v>
+      </c>
+      <c r="N17" t="n">
+        <v>45295.04218553174</v>
+      </c>
+      <c r="O17" t="n">
+        <v>0</v>
+      </c>
+      <c r="P17" t="n">
+        <v>45295.04218553174</v>
+      </c>
+      <c r="Q17" t="n">
+        <v>45290.34926299912</v>
+      </c>
+      <c r="R17" t="n">
+        <v>0</v>
+      </c>
+      <c r="S17" t="n">
+        <v>0</v>
+      </c>
+      <c r="T17" t="n">
+        <v>0</v>
+      </c>
+      <c r="U17" t="n">
+        <v>4.692922532634418</v>
+      </c>
+      <c r="V17" t="n">
+        <v>3.075000047683716</v>
+      </c>
+      <c r="W17" t="n">
+        <v>42575562.54061422</v>
+      </c>
+      <c r="X17" t="n">
+        <v>42575562.54061422</v>
+      </c>
+      <c r="Y17" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z17" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA17" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC17" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD17" t="inlineStr">
+        <is>
+          <t>el_price_150_costs</t>
+        </is>
+      </c>
+      <c r="AE17" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_WtE\raw_results\CaL\20260128144230_el_price_150_costs</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>37680267.05113474</v>
+      </c>
+      <c r="B18" t="n">
+        <v>30920004.27095176</v>
+      </c>
+      <c r="C18" t="n">
+        <v>4371031.010497759</v>
+      </c>
+      <c r="D18" t="n">
+        <v>23243173.15400708</v>
+      </c>
+      <c r="E18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F18" t="n">
+        <v>54163177.42495884</v>
+      </c>
+      <c r="G18" t="n">
+        <v>4371031.010497759</v>
+      </c>
+      <c r="H18" t="n">
+        <v>2583505.769331105</v>
+      </c>
+      <c r="I18" t="n">
+        <v>-34363856.15648095</v>
+      </c>
+      <c r="J18" t="n">
+        <v>0</v>
+      </c>
+      <c r="K18" t="n">
+        <v>0</v>
+      </c>
+      <c r="L18" t="n">
+        <v>10926409.00282798</v>
+      </c>
+      <c r="M18" t="n">
+        <v>37680267.05113474</v>
+      </c>
+      <c r="N18" t="n">
+        <v>43710.37622015406</v>
+      </c>
+      <c r="O18" t="n">
+        <v>0</v>
+      </c>
+      <c r="P18" t="n">
+        <v>43710.37622015406</v>
+      </c>
+      <c r="Q18" t="n">
+        <v>43705.63601131194</v>
+      </c>
+      <c r="R18" t="n">
+        <v>0</v>
+      </c>
+      <c r="S18" t="n">
+        <v>0</v>
+      </c>
+      <c r="T18" t="n">
+        <v>0</v>
+      </c>
+      <c r="U18" t="n">
+        <v>4.740208842091318</v>
+      </c>
+      <c r="V18" t="n">
+        <v>2.917999982833862</v>
+      </c>
+      <c r="W18" t="n">
+        <v>37680267.05113474</v>
+      </c>
+      <c r="X18" t="n">
+        <v>37680267.05113474</v>
+      </c>
+      <c r="Y18" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z18" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA18" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB18" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC18" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD18" t="inlineStr">
+        <is>
+          <t>el_price_175_costs</t>
+        </is>
+      </c>
+      <c r="AE18" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_WtE\raw_results\CaL\20260128144446_el_price_175_costs</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>56705688.96974421</v>
+      </c>
+      <c r="B19" t="n">
+        <v>23602309.58151861</v>
+      </c>
+      <c r="C19" t="n">
+        <v>3675691.270406743</v>
+      </c>
+      <c r="D19" t="n">
+        <v>17966626.69030973</v>
+      </c>
+      <c r="E19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F19" t="n">
+        <v>41568936.27182833</v>
+      </c>
+      <c r="G19" t="n">
+        <v>3675691.270406743</v>
+      </c>
+      <c r="H19" t="n">
+        <v>1846745.394398591</v>
+      </c>
+      <c r="I19" t="n">
+        <v>-12877164.53350351</v>
+      </c>
+      <c r="J19" t="n">
+        <v>0</v>
+      </c>
+      <c r="K19" t="n">
+        <v>0</v>
+      </c>
+      <c r="L19" t="n">
+        <v>22491480.56661404</v>
+      </c>
+      <c r="M19" t="n">
+        <v>56705688.96974421</v>
+      </c>
+      <c r="N19" t="n">
+        <v>89969.36363936203</v>
+      </c>
+      <c r="O19" t="n">
+        <v>0</v>
+      </c>
+      <c r="P19" t="n">
+        <v>89969.36363936203</v>
+      </c>
+      <c r="Q19" t="n">
+        <v>89965.92226645617</v>
+      </c>
+      <c r="R19" t="n">
+        <v>0</v>
+      </c>
+      <c r="S19" t="n">
+        <v>0</v>
+      </c>
+      <c r="T19" t="n">
+        <v>0</v>
+      </c>
+      <c r="U19" t="n">
+        <v>3.441372905900046</v>
+      </c>
+      <c r="V19" t="n">
+        <v>3.47599983215332</v>
+      </c>
+      <c r="W19" t="n">
+        <v>56705688.96974421</v>
+      </c>
+      <c r="X19" t="n">
+        <v>56705688.96974421</v>
+      </c>
+      <c r="Y19" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z19" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA19" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB19" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC19" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD19" t="inlineStr">
+        <is>
+          <t>el_price_75_costs</t>
+        </is>
+      </c>
+      <c r="AE19" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_WtE\raw_results\CaL\20260128151650_el_price_75_costs</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>52229394.09413296</v>
+      </c>
+      <c r="B20" t="n">
+        <v>28580992.5973305</v>
+      </c>
+      <c r="C20" t="n">
+        <v>4148774.160734102</v>
+      </c>
+      <c r="D20" t="n">
+        <v>21569232.87215166</v>
+      </c>
+      <c r="E20" t="n">
+        <v>0</v>
+      </c>
+      <c r="F20" t="n">
+        <v>50150225.46948216</v>
+      </c>
+      <c r="G20" t="n">
+        <v>4148774.160734102</v>
+      </c>
+      <c r="H20" t="n">
+        <v>2330102.374502039</v>
+      </c>
+      <c r="I20" t="n">
+        <v>-18838351.33481684</v>
+      </c>
+      <c r="J20" t="n">
+        <v>0</v>
+      </c>
+      <c r="K20" t="n">
+        <v>0</v>
+      </c>
+      <c r="L20" t="n">
+        <v>14438643.42423149</v>
+      </c>
+      <c r="M20" t="n">
+        <v>52229394.09413296</v>
+      </c>
+      <c r="N20" t="n">
+        <v>57758.91587147661</v>
+      </c>
+      <c r="O20" t="n">
+        <v>0</v>
+      </c>
+      <c r="P20" t="n">
+        <v>57758.91587147661</v>
+      </c>
+      <c r="Q20" t="n">
+        <v>57754.57369692596</v>
+      </c>
+      <c r="R20" t="n">
+        <v>0</v>
+      </c>
+      <c r="S20" t="n">
+        <v>0</v>
+      </c>
+      <c r="T20" t="n">
+        <v>0</v>
+      </c>
+      <c r="U20" t="n">
+        <v>4.34217455063829</v>
+      </c>
+      <c r="V20" t="n">
+        <v>3.396999835968018</v>
+      </c>
+      <c r="W20" t="n">
+        <v>52229394.09413296</v>
+      </c>
+      <c r="X20" t="n">
+        <v>52229394.09413296</v>
+      </c>
+      <c r="Y20" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z20" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA20" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB20" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC20" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD20" t="inlineStr">
+        <is>
+          <t>el_price_100_costs</t>
+        </is>
+      </c>
+      <c r="AE20" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_WtE\raw_results\CaL\20260128151911_el_price_100_costs</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>47436854.16685127</v>
+      </c>
+      <c r="B21" t="n">
+        <v>30170466.41311156</v>
+      </c>
+      <c r="C21" t="n">
+        <v>4299808.654089317</v>
+      </c>
+      <c r="D21" t="n">
+        <v>22711260.94737182</v>
+      </c>
+      <c r="E21" t="n">
+        <v>0</v>
+      </c>
+      <c r="F21" t="n">
+        <v>52881727.36048338</v>
+      </c>
+      <c r="G21" t="n">
+        <v>4299808.654089317</v>
+      </c>
+      <c r="H21" t="n">
+        <v>2483596.055394794</v>
+      </c>
+      <c r="I21" t="n">
+        <v>-24200253.56808047</v>
+      </c>
+      <c r="J21" t="n">
+        <v>0</v>
+      </c>
+      <c r="K21" t="n">
+        <v>0</v>
+      </c>
+      <c r="L21" t="n">
+        <v>11971975.66496425</v>
+      </c>
+      <c r="M21" t="n">
+        <v>47436854.16685127</v>
+      </c>
+      <c r="N21" t="n">
+        <v>47892.52141683055</v>
+      </c>
+      <c r="O21" t="n">
+        <v>0</v>
+      </c>
+      <c r="P21" t="n">
+        <v>47892.52141683055</v>
+      </c>
+      <c r="Q21" t="n">
+        <v>47887.90265985703</v>
+      </c>
+      <c r="R21" t="n">
+        <v>0</v>
+      </c>
+      <c r="S21" t="n">
+        <v>0</v>
+      </c>
+      <c r="T21" t="n">
+        <v>0</v>
+      </c>
+      <c r="U21" t="n">
+        <v>4.618756973548098</v>
+      </c>
+      <c r="V21" t="n">
+        <v>3.236999988555908</v>
+      </c>
+      <c r="W21" t="n">
+        <v>47436854.16685127</v>
+      </c>
+      <c r="X21" t="n">
+        <v>47436854.16685127</v>
+      </c>
+      <c r="Y21" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z21" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA21" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB21" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC21" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD21" t="inlineStr">
+        <is>
+          <t>el_price_125_costs</t>
+        </is>
+      </c>
+      <c r="AE21" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_WtE\raw_results\CaL\20260128152141_el_price_125_costs</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>42575562.54061422</v>
+      </c>
+      <c r="B22" t="n">
+        <v>30620008.39546236</v>
+      </c>
+      <c r="C22" t="n">
+        <v>4342524.894440144</v>
+      </c>
+      <c r="D22" t="n">
+        <v>23031257.4414313</v>
+      </c>
+      <c r="E22" t="n">
+        <v>0</v>
+      </c>
+      <c r="F22" t="n">
+        <v>53651265.83689366</v>
+      </c>
+      <c r="G22" t="n">
+        <v>4342524.894440144</v>
+      </c>
+      <c r="H22" t="n">
+        <v>2535175.660100587</v>
+      </c>
+      <c r="I22" t="n">
+        <v>-29275991.16656995</v>
+      </c>
+      <c r="J22" t="n">
+        <v>0</v>
+      </c>
+      <c r="K22" t="n">
+        <v>0</v>
+      </c>
+      <c r="L22" t="n">
+        <v>11322587.31574978</v>
+      </c>
+      <c r="M22" t="n">
+        <v>42575562.54061422</v>
+      </c>
+      <c r="N22" t="n">
+        <v>45295.04218553174</v>
+      </c>
+      <c r="O22" t="n">
+        <v>0</v>
+      </c>
+      <c r="P22" t="n">
+        <v>45295.04218553174</v>
+      </c>
+      <c r="Q22" t="n">
+        <v>45290.34926299912</v>
+      </c>
+      <c r="R22" t="n">
+        <v>0</v>
+      </c>
+      <c r="S22" t="n">
+        <v>0</v>
+      </c>
+      <c r="T22" t="n">
+        <v>0</v>
+      </c>
+      <c r="U22" t="n">
+        <v>4.692922532634418</v>
+      </c>
+      <c r="V22" t="n">
+        <v>3.314000129699707</v>
+      </c>
+      <c r="W22" t="n">
+        <v>42575562.54061422</v>
+      </c>
+      <c r="X22" t="n">
+        <v>42575562.54061422</v>
+      </c>
+      <c r="Y22" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z22" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA22" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB22" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC22" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD22" t="inlineStr">
+        <is>
+          <t>el_price_150_costs</t>
+        </is>
+      </c>
+      <c r="AE22" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_WtE\raw_results\CaL\20260128152410_el_price_150_costs</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>37680267.05113474</v>
+      </c>
+      <c r="B23" t="n">
+        <v>30920004.27095176</v>
+      </c>
+      <c r="C23" t="n">
+        <v>4371031.010497759</v>
+      </c>
+      <c r="D23" t="n">
+        <v>23243173.15400708</v>
+      </c>
+      <c r="E23" t="n">
+        <v>0</v>
+      </c>
+      <c r="F23" t="n">
+        <v>54163177.42495884</v>
+      </c>
+      <c r="G23" t="n">
+        <v>4371031.010497759</v>
+      </c>
+      <c r="H23" t="n">
+        <v>2583505.769331105</v>
+      </c>
+      <c r="I23" t="n">
+        <v>-34363856.15648095</v>
+      </c>
+      <c r="J23" t="n">
+        <v>0</v>
+      </c>
+      <c r="K23" t="n">
+        <v>0</v>
+      </c>
+      <c r="L23" t="n">
+        <v>10926409.00282798</v>
+      </c>
+      <c r="M23" t="n">
+        <v>37680267.05113474</v>
+      </c>
+      <c r="N23" t="n">
+        <v>43710.37622015406</v>
+      </c>
+      <c r="O23" t="n">
+        <v>0</v>
+      </c>
+      <c r="P23" t="n">
+        <v>43710.37622015406</v>
+      </c>
+      <c r="Q23" t="n">
+        <v>43705.63601131194</v>
+      </c>
+      <c r="R23" t="n">
+        <v>0</v>
+      </c>
+      <c r="S23" t="n">
+        <v>0</v>
+      </c>
+      <c r="T23" t="n">
+        <v>0</v>
+      </c>
+      <c r="U23" t="n">
+        <v>4.740208842091318</v>
+      </c>
+      <c r="V23" t="n">
+        <v>3.329999923706055</v>
+      </c>
+      <c r="W23" t="n">
+        <v>37680267.05113474</v>
+      </c>
+      <c r="X23" t="n">
+        <v>37680267.05113474</v>
+      </c>
+      <c r="Y23" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z23" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA23" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB23" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC23" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD23" t="inlineStr">
+        <is>
+          <t>el_price_175_costs</t>
+        </is>
+      </c>
+      <c r="AE23" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_WtE\raw_results\CaL\20260128152627_el_price_175_costs</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
results cal and tech selection wte
</commit_message>
<xml_diff>
--- a/dataCaseStudy_WtE/raw_results/CaL/Summary.xlsx
+++ b/dataCaseStudy_WtE/raw_results/CaL/Summary.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE23"/>
+  <dimension ref="A1:AE33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2848,6 +2848,1036 @@
       <c r="AE23" t="inlineStr">
         <is>
           <t>dataCaseStudy_WtE\raw_results\CaL\20260128152627_el_price_175_costs</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>56705650.20608237</v>
+      </c>
+      <c r="B24" t="n">
+        <v>23602309.58151861</v>
+      </c>
+      <c r="C24" t="n">
+        <v>3675691.270406743</v>
+      </c>
+      <c r="D24" t="n">
+        <v>17966626.69030973</v>
+      </c>
+      <c r="E24" t="n">
+        <v>0</v>
+      </c>
+      <c r="F24" t="n">
+        <v>41568936.27182833</v>
+      </c>
+      <c r="G24" t="n">
+        <v>3675691.270406743</v>
+      </c>
+      <c r="H24" t="n">
+        <v>1846706.630736768</v>
+      </c>
+      <c r="I24" t="n">
+        <v>-12877164.53350351</v>
+      </c>
+      <c r="J24" t="n">
+        <v>0</v>
+      </c>
+      <c r="K24" t="n">
+        <v>0</v>
+      </c>
+      <c r="L24" t="n">
+        <v>22491480.56661404</v>
+      </c>
+      <c r="M24" t="n">
+        <v>56705650.20608237</v>
+      </c>
+      <c r="N24" t="n">
+        <v>89969.36363936203</v>
+      </c>
+      <c r="O24" t="n">
+        <v>0</v>
+      </c>
+      <c r="P24" t="n">
+        <v>89969.36363936203</v>
+      </c>
+      <c r="Q24" t="n">
+        <v>89965.92226645617</v>
+      </c>
+      <c r="R24" t="n">
+        <v>0</v>
+      </c>
+      <c r="S24" t="n">
+        <v>0</v>
+      </c>
+      <c r="T24" t="n">
+        <v>0</v>
+      </c>
+      <c r="U24" t="n">
+        <v>3.441372905900046</v>
+      </c>
+      <c r="V24" t="n">
+        <v>3.086999893188477</v>
+      </c>
+      <c r="W24" t="n">
+        <v>56705650.20608237</v>
+      </c>
+      <c r="X24" t="n">
+        <v>56705650.20608237</v>
+      </c>
+      <c r="Y24" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z24" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA24" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB24" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC24" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD24" t="inlineStr">
+        <is>
+          <t>el_price_75_costs</t>
+        </is>
+      </c>
+      <c r="AE24" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_WtE\raw_results\CaL\20260128185442_el_price_75_costs</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>52229355.33047114</v>
+      </c>
+      <c r="B25" t="n">
+        <v>28580992.5973305</v>
+      </c>
+      <c r="C25" t="n">
+        <v>4148774.160734102</v>
+      </c>
+      <c r="D25" t="n">
+        <v>21569232.87215166</v>
+      </c>
+      <c r="E25" t="n">
+        <v>0</v>
+      </c>
+      <c r="F25" t="n">
+        <v>50150225.46948216</v>
+      </c>
+      <c r="G25" t="n">
+        <v>4148774.160734102</v>
+      </c>
+      <c r="H25" t="n">
+        <v>2330063.610840216</v>
+      </c>
+      <c r="I25" t="n">
+        <v>-18838351.33481684</v>
+      </c>
+      <c r="J25" t="n">
+        <v>0</v>
+      </c>
+      <c r="K25" t="n">
+        <v>0</v>
+      </c>
+      <c r="L25" t="n">
+        <v>14438643.42423149</v>
+      </c>
+      <c r="M25" t="n">
+        <v>52229355.33047114</v>
+      </c>
+      <c r="N25" t="n">
+        <v>57758.91587147661</v>
+      </c>
+      <c r="O25" t="n">
+        <v>0</v>
+      </c>
+      <c r="P25" t="n">
+        <v>57758.91587147661</v>
+      </c>
+      <c r="Q25" t="n">
+        <v>57754.57369692596</v>
+      </c>
+      <c r="R25" t="n">
+        <v>0</v>
+      </c>
+      <c r="S25" t="n">
+        <v>0</v>
+      </c>
+      <c r="T25" t="n">
+        <v>0</v>
+      </c>
+      <c r="U25" t="n">
+        <v>4.34217455063829</v>
+      </c>
+      <c r="V25" t="n">
+        <v>2.950000047683716</v>
+      </c>
+      <c r="W25" t="n">
+        <v>52229355.33047114</v>
+      </c>
+      <c r="X25" t="n">
+        <v>52229355.33047114</v>
+      </c>
+      <c r="Y25" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z25" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA25" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC25" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD25" t="inlineStr">
+        <is>
+          <t>el_price_100_costs</t>
+        </is>
+      </c>
+      <c r="AE25" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_WtE\raw_results\CaL\20260128185701_el_price_100_costs</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>47434341.81768903</v>
+      </c>
+      <c r="B26" t="n">
+        <v>30170466.41311156</v>
+      </c>
+      <c r="C26" t="n">
+        <v>4299808.654089317</v>
+      </c>
+      <c r="D26" t="n">
+        <v>22711260.94737182</v>
+      </c>
+      <c r="E26" t="n">
+        <v>0</v>
+      </c>
+      <c r="F26" t="n">
+        <v>52881727.36048338</v>
+      </c>
+      <c r="G26" t="n">
+        <v>4299808.654089317</v>
+      </c>
+      <c r="H26" t="n">
+        <v>2488561.166745042</v>
+      </c>
+      <c r="I26" t="n">
+        <v>-24217404.64018829</v>
+      </c>
+      <c r="J26" t="n">
+        <v>0</v>
+      </c>
+      <c r="K26" t="n">
+        <v>0</v>
+      </c>
+      <c r="L26" t="n">
+        <v>11981649.27655958</v>
+      </c>
+      <c r="M26" t="n">
+        <v>47434341.81768903</v>
+      </c>
+      <c r="N26" t="n">
+        <v>47931.21586321186</v>
+      </c>
+      <c r="O26" t="n">
+        <v>0</v>
+      </c>
+      <c r="P26" t="n">
+        <v>47931.21586321186</v>
+      </c>
+      <c r="Q26" t="n">
+        <v>47926.59710623833</v>
+      </c>
+      <c r="R26" t="n">
+        <v>0</v>
+      </c>
+      <c r="S26" t="n">
+        <v>0</v>
+      </c>
+      <c r="T26" t="n">
+        <v>0</v>
+      </c>
+      <c r="U26" t="n">
+        <v>4.618756973548098</v>
+      </c>
+      <c r="V26" t="n">
+        <v>2.996999979019165</v>
+      </c>
+      <c r="W26" t="n">
+        <v>47434341.81768903</v>
+      </c>
+      <c r="X26" t="n">
+        <v>47434341.81768903</v>
+      </c>
+      <c r="Y26" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z26" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA26" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB26" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC26" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD26" t="inlineStr">
+        <is>
+          <t>el_price_125_costs</t>
+        </is>
+      </c>
+      <c r="AE26" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_WtE\raw_results\CaL\20260128185926_el_price_125_costs</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>42569275.14786529</v>
+      </c>
+      <c r="B27" t="n">
+        <v>30620008.39546236</v>
+      </c>
+      <c r="C27" t="n">
+        <v>4342524.894440144</v>
+      </c>
+      <c r="D27" t="n">
+        <v>23031257.4414313</v>
+      </c>
+      <c r="E27" t="n">
+        <v>0</v>
+      </c>
+      <c r="F27" t="n">
+        <v>53651265.83689366</v>
+      </c>
+      <c r="G27" t="n">
+        <v>4342524.894440144</v>
+      </c>
+      <c r="H27" t="n">
+        <v>2543368.416960416</v>
+      </c>
+      <c r="I27" t="n">
+        <v>-29309662.41969334</v>
+      </c>
+      <c r="J27" t="n">
+        <v>0</v>
+      </c>
+      <c r="K27" t="n">
+        <v>0</v>
+      </c>
+      <c r="L27" t="n">
+        <v>11341778.4192644</v>
+      </c>
+      <c r="M27" t="n">
+        <v>42569275.14786529</v>
+      </c>
+      <c r="N27" t="n">
+        <v>45371.80659959024</v>
+      </c>
+      <c r="O27" t="n">
+        <v>0</v>
+      </c>
+      <c r="P27" t="n">
+        <v>45371.80659959024</v>
+      </c>
+      <c r="Q27" t="n">
+        <v>45367.11367705761</v>
+      </c>
+      <c r="R27" t="n">
+        <v>0</v>
+      </c>
+      <c r="S27" t="n">
+        <v>0</v>
+      </c>
+      <c r="T27" t="n">
+        <v>0</v>
+      </c>
+      <c r="U27" t="n">
+        <v>4.692922532634418</v>
+      </c>
+      <c r="V27" t="n">
+        <v>3.069999933242798</v>
+      </c>
+      <c r="W27" t="n">
+        <v>42569275.14786529</v>
+      </c>
+      <c r="X27" t="n">
+        <v>42569275.14786529</v>
+      </c>
+      <c r="Y27" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z27" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA27" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB27" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC27" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD27" t="inlineStr">
+        <is>
+          <t>el_price_150_costs</t>
+        </is>
+      </c>
+      <c r="AE27" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_WtE\raw_results\CaL\20260128190155_el_price_150_costs</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>37663103.6152001</v>
+      </c>
+      <c r="B28" t="n">
+        <v>30920004.27095176</v>
+      </c>
+      <c r="C28" t="n">
+        <v>4371031.010497759</v>
+      </c>
+      <c r="D28" t="n">
+        <v>23243173.15400708</v>
+      </c>
+      <c r="E28" t="n">
+        <v>0</v>
+      </c>
+      <c r="F28" t="n">
+        <v>54163177.42495884</v>
+      </c>
+      <c r="G28" t="n">
+        <v>4371031.010497759</v>
+      </c>
+      <c r="H28" t="n">
+        <v>2633349.881300342</v>
+      </c>
+      <c r="I28" t="n">
+        <v>-34523115.31161098</v>
+      </c>
+      <c r="J28" t="n">
+        <v>0</v>
+      </c>
+      <c r="K28" t="n">
+        <v>0</v>
+      </c>
+      <c r="L28" t="n">
+        <v>11018660.61005414</v>
+      </c>
+      <c r="M28" t="n">
+        <v>37663103.6152001</v>
+      </c>
+      <c r="N28" t="n">
+        <v>44079.38264905868</v>
+      </c>
+      <c r="O28" t="n">
+        <v>0</v>
+      </c>
+      <c r="P28" t="n">
+        <v>44079.38264905868</v>
+      </c>
+      <c r="Q28" t="n">
+        <v>44074.64244021656</v>
+      </c>
+      <c r="R28" t="n">
+        <v>0</v>
+      </c>
+      <c r="S28" t="n">
+        <v>0</v>
+      </c>
+      <c r="T28" t="n">
+        <v>0</v>
+      </c>
+      <c r="U28" t="n">
+        <v>4.740208842091318</v>
+      </c>
+      <c r="V28" t="n">
+        <v>3.020999908447266</v>
+      </c>
+      <c r="W28" t="n">
+        <v>37663103.6152001</v>
+      </c>
+      <c r="X28" t="n">
+        <v>37663103.6152001</v>
+      </c>
+      <c r="Y28" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z28" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA28" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC28" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD28" t="inlineStr">
+        <is>
+          <t>el_price_175_costs</t>
+        </is>
+      </c>
+      <c r="AE28" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_WtE\raw_results\CaL\20260128190415_el_price_175_costs</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>54551112.11099866</v>
+      </c>
+      <c r="B29" t="n">
+        <v>31090637.89623569</v>
+      </c>
+      <c r="C29" t="n">
+        <v>4387244.906497965</v>
+      </c>
+      <c r="D29" t="n">
+        <v>23362895.97562808</v>
+      </c>
+      <c r="E29" t="n">
+        <v>0</v>
+      </c>
+      <c r="F29" t="n">
+        <v>54453533.87186377</v>
+      </c>
+      <c r="G29" t="n">
+        <v>4387244.906497965</v>
+      </c>
+      <c r="H29" t="n">
+        <v>2557523.584690922</v>
+      </c>
+      <c r="I29" t="n">
+        <v>-19626895.50306778</v>
+      </c>
+      <c r="J29" t="n">
+        <v>0</v>
+      </c>
+      <c r="K29" t="n">
+        <v>0</v>
+      </c>
+      <c r="L29" t="n">
+        <v>12779705.25101378</v>
+      </c>
+      <c r="M29" t="n">
+        <v>54551112.11099866</v>
+      </c>
+      <c r="N29" t="n">
+        <v>42603.78350836707</v>
+      </c>
+      <c r="O29" t="n">
+        <v>0</v>
+      </c>
+      <c r="P29" t="n">
+        <v>42603.78350836707</v>
+      </c>
+      <c r="Q29" t="n">
+        <v>42599.01750337926</v>
+      </c>
+      <c r="R29" t="n">
+        <v>0</v>
+      </c>
+      <c r="S29" t="n">
+        <v>0</v>
+      </c>
+      <c r="T29" t="n">
+        <v>0</v>
+      </c>
+      <c r="U29" t="n">
+        <v>4.766004987808616</v>
+      </c>
+      <c r="V29" t="n">
+        <v>3.843999862670898</v>
+      </c>
+      <c r="W29" t="n">
+        <v>54551112.11099866</v>
+      </c>
+      <c r="X29" t="n">
+        <v>54551112.11099866</v>
+      </c>
+      <c r="Y29" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z29" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA29" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB29" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC29" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD29" t="inlineStr">
+        <is>
+          <t>el_price_100_costs</t>
+        </is>
+      </c>
+      <c r="AE29" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_WtE\raw_results\CaL\20260202162700_el_price_100_costs</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>49637638.00808052</v>
+      </c>
+      <c r="B30" t="n">
+        <v>31289233.83448502</v>
+      </c>
+      <c r="C30" t="n">
+        <v>4406115.828823382</v>
+      </c>
+      <c r="D30" t="n">
+        <v>23501390.40939506</v>
+      </c>
+      <c r="E30" t="n">
+        <v>0</v>
+      </c>
+      <c r="F30" t="n">
+        <v>54790624.24388008</v>
+      </c>
+      <c r="G30" t="n">
+        <v>4406115.828823382</v>
+      </c>
+      <c r="H30" t="n">
+        <v>2573017.655303521</v>
+      </c>
+      <c r="I30" t="n">
+        <v>-24602063.2855968</v>
+      </c>
+      <c r="J30" t="n">
+        <v>0</v>
+      </c>
+      <c r="K30" t="n">
+        <v>0</v>
+      </c>
+      <c r="L30" t="n">
+        <v>12469943.56567033</v>
+      </c>
+      <c r="M30" t="n">
+        <v>49637638.00808052</v>
+      </c>
+      <c r="N30" t="n">
+        <v>41571.27343253568</v>
+      </c>
+      <c r="O30" t="n">
+        <v>0</v>
+      </c>
+      <c r="P30" t="n">
+        <v>41571.27343253568</v>
+      </c>
+      <c r="Q30" t="n">
+        <v>41566.47855223444</v>
+      </c>
+      <c r="R30" t="n">
+        <v>0</v>
+      </c>
+      <c r="S30" t="n">
+        <v>0</v>
+      </c>
+      <c r="T30" t="n">
+        <v>0</v>
+      </c>
+      <c r="U30" t="n">
+        <v>4.794880301223074</v>
+      </c>
+      <c r="V30" t="n">
+        <v>2.952000141143799</v>
+      </c>
+      <c r="W30" t="n">
+        <v>49637638.00808052</v>
+      </c>
+      <c r="X30" t="n">
+        <v>49637638.00808052</v>
+      </c>
+      <c r="Y30" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z30" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA30" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC30" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD30" t="inlineStr">
+        <is>
+          <t>el_price_125_costs</t>
+        </is>
+      </c>
+      <c r="AE30" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_WtE\raw_results\CaL\20260202162918_el_price_125_costs</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>44708664.97812186</v>
+      </c>
+      <c r="B31" t="n">
+        <v>31479609.3409155</v>
+      </c>
+      <c r="C31" t="n">
+        <v>4424205.631798112</v>
+      </c>
+      <c r="D31" t="n">
+        <v>23633332.99817676</v>
+      </c>
+      <c r="E31" t="n">
+        <v>0</v>
+      </c>
+      <c r="F31" t="n">
+        <v>55112942.33909227</v>
+      </c>
+      <c r="G31" t="n">
+        <v>4424205.631798112</v>
+      </c>
+      <c r="H31" t="n">
+        <v>2598877.293728911</v>
+      </c>
+      <c r="I31" t="n">
+        <v>-29628363.36563013</v>
+      </c>
+      <c r="J31" t="n">
+        <v>0</v>
+      </c>
+      <c r="K31" t="n">
+        <v>0</v>
+      </c>
+      <c r="L31" t="n">
+        <v>12201003.07913271</v>
+      </c>
+      <c r="M31" t="n">
+        <v>44708664.97812186</v>
+      </c>
+      <c r="N31" t="n">
+        <v>40674.83171475254</v>
+      </c>
+      <c r="O31" t="n">
+        <v>0</v>
+      </c>
+      <c r="P31" t="n">
+        <v>40674.83171475254</v>
+      </c>
+      <c r="Q31" t="n">
+        <v>40670.01026377569</v>
+      </c>
+      <c r="R31" t="n">
+        <v>0</v>
+      </c>
+      <c r="S31" t="n">
+        <v>0</v>
+      </c>
+      <c r="T31" t="n">
+        <v>0</v>
+      </c>
+      <c r="U31" t="n">
+        <v>4.82145097683823</v>
+      </c>
+      <c r="V31" t="n">
+        <v>3.091000080108643</v>
+      </c>
+      <c r="W31" t="n">
+        <v>44708664.97812186</v>
+      </c>
+      <c r="X31" t="n">
+        <v>44708664.97812186</v>
+      </c>
+      <c r="Y31" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z31" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA31" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC31" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD31" t="inlineStr">
+        <is>
+          <t>el_price_150_costs</t>
+        </is>
+      </c>
+      <c r="AE31" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_WtE\raw_results\CaL\20260202163141_el_price_150_costs</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>39763317.70086691</v>
+      </c>
+      <c r="B32" t="n">
+        <v>31644675.4328307</v>
+      </c>
+      <c r="C32" t="n">
+        <v>4439890.491350382</v>
+      </c>
+      <c r="D32" t="n">
+        <v>23747074.321913</v>
+      </c>
+      <c r="E32" t="n">
+        <v>0</v>
+      </c>
+      <c r="F32" t="n">
+        <v>55391749.75474371</v>
+      </c>
+      <c r="G32" t="n">
+        <v>4439890.491350382</v>
+      </c>
+      <c r="H32" t="n">
+        <v>2622589.083656741</v>
+      </c>
+      <c r="I32" t="n">
+        <v>-34670775.568021</v>
+      </c>
+      <c r="J32" t="n">
+        <v>0</v>
+      </c>
+      <c r="K32" t="n">
+        <v>0</v>
+      </c>
+      <c r="L32" t="n">
+        <v>11979863.93913708</v>
+      </c>
+      <c r="M32" t="n">
+        <v>39763317.70086691</v>
+      </c>
+      <c r="N32" t="n">
+        <v>39937.72339224516</v>
+      </c>
+      <c r="O32" t="n">
+        <v>0</v>
+      </c>
+      <c r="P32" t="n">
+        <v>39937.72339224516</v>
+      </c>
+      <c r="Q32" t="n">
+        <v>39932.87979712251</v>
+      </c>
+      <c r="R32" t="n">
+        <v>0</v>
+      </c>
+      <c r="S32" t="n">
+        <v>0</v>
+      </c>
+      <c r="T32" t="n">
+        <v>0</v>
+      </c>
+      <c r="U32" t="n">
+        <v>4.843595121557295</v>
+      </c>
+      <c r="V32" t="n">
+        <v>2.934999942779541</v>
+      </c>
+      <c r="W32" t="n">
+        <v>39763317.70086691</v>
+      </c>
+      <c r="X32" t="n">
+        <v>39763317.70086691</v>
+      </c>
+      <c r="Y32" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z32" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA32" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC32" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD32" t="inlineStr">
+        <is>
+          <t>el_price_175_costs</t>
+        </is>
+      </c>
+      <c r="AE32" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_WtE\raw_results\CaL\20260202163409_el_price_175_costs</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>34802702.85566229</v>
+      </c>
+      <c r="B33" t="n">
+        <v>31770005.71753078</v>
+      </c>
+      <c r="C33" t="n">
+        <v>4451799.587218337</v>
+      </c>
+      <c r="D33" t="n">
+        <v>23832960.21389318</v>
+      </c>
+      <c r="E33" t="n">
+        <v>0</v>
+      </c>
+      <c r="F33" t="n">
+        <v>55602965.93142396</v>
+      </c>
+      <c r="G33" t="n">
+        <v>4451799.587218337</v>
+      </c>
+      <c r="H33" t="n">
+        <v>2656059.808211191</v>
+      </c>
+      <c r="I33" t="n">
+        <v>-39748919.55638661</v>
+      </c>
+      <c r="J33" t="n">
+        <v>0</v>
+      </c>
+      <c r="K33" t="n">
+        <v>0</v>
+      </c>
+      <c r="L33" t="n">
+        <v>11840797.08519541</v>
+      </c>
+      <c r="M33" t="n">
+        <v>34802702.85566229</v>
+      </c>
+      <c r="N33" t="n">
+        <v>39474.18338279358</v>
+      </c>
+      <c r="O33" t="n">
+        <v>0</v>
+      </c>
+      <c r="P33" t="n">
+        <v>39474.18338279358</v>
+      </c>
+      <c r="Q33" t="n">
+        <v>39469.32361731802</v>
+      </c>
+      <c r="R33" t="n">
+        <v>0</v>
+      </c>
+      <c r="S33" t="n">
+        <v>0</v>
+      </c>
+      <c r="T33" t="n">
+        <v>0</v>
+      </c>
+      <c r="U33" t="n">
+        <v>4.859765475555238</v>
+      </c>
+      <c r="V33" t="n">
+        <v>2.851000070571899</v>
+      </c>
+      <c r="W33" t="n">
+        <v>34802702.85566229</v>
+      </c>
+      <c r="X33" t="n">
+        <v>34802702.85566229</v>
+      </c>
+      <c r="Y33" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z33" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA33" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC33" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD33" t="inlineStr">
+        <is>
+          <t>el_price_200_costs</t>
+        </is>
+      </c>
+      <c r="AE33" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_WtE\raw_results\CaL\20260202163626_el_price_200_costs</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
results cal (tax at 250) and tech selection wte
</commit_message>
<xml_diff>
--- a/dataCaseStudy_WtE/raw_results/CaL/Summary.xlsx
+++ b/dataCaseStudy_WtE/raw_results/CaL/Summary.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE33"/>
+  <dimension ref="A1:AE39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3878,6 +3878,624 @@
       <c r="AE33" t="inlineStr">
         <is>
           <t>dataCaseStudy_WtE\raw_results\CaL\20260202163626_el_price_200_costs</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>57367656.50849163</v>
+      </c>
+      <c r="B34" t="n">
+        <v>0</v>
+      </c>
+      <c r="C34" t="n">
+        <v>0</v>
+      </c>
+      <c r="D34" t="n">
+        <v>1500000</v>
+      </c>
+      <c r="E34" t="n">
+        <v>0</v>
+      </c>
+      <c r="F34" t="n">
+        <v>1500000</v>
+      </c>
+      <c r="G34" t="n">
+        <v>0</v>
+      </c>
+      <c r="H34" t="n">
+        <v>155.0546472912404</v>
+      </c>
+      <c r="I34" t="n">
+        <v>-8039812.913946624</v>
+      </c>
+      <c r="J34" t="n">
+        <v>0</v>
+      </c>
+      <c r="K34" t="n">
+        <v>0</v>
+      </c>
+      <c r="L34" t="n">
+        <v>63907314.36779096</v>
+      </c>
+      <c r="M34" t="n">
+        <v>57367656.50849163</v>
+      </c>
+      <c r="N34" t="n">
+        <v>213024.3812259698</v>
+      </c>
+      <c r="O34" t="n">
+        <v>0</v>
+      </c>
+      <c r="P34" t="n">
+        <v>213024.3812259698</v>
+      </c>
+      <c r="Q34" t="n">
+        <v>213024.3812259698</v>
+      </c>
+      <c r="R34" t="n">
+        <v>0</v>
+      </c>
+      <c r="S34" t="n">
+        <v>0</v>
+      </c>
+      <c r="T34" t="n">
+        <v>0</v>
+      </c>
+      <c r="U34" t="n">
+        <v>0</v>
+      </c>
+      <c r="V34" t="n">
+        <v>4.161999940872192</v>
+      </c>
+      <c r="W34" t="n">
+        <v>57367656.50849163</v>
+      </c>
+      <c r="X34" t="n">
+        <v>57367656.50849163</v>
+      </c>
+      <c r="Y34" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z34" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA34" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB34" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC34" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD34" t="inlineStr">
+        <is>
+          <t>el_price_75_costs</t>
+        </is>
+      </c>
+      <c r="AE34" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_WtE\raw_results\CaL\20260203181303_el_price_75_costs</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>54551112.11099866</v>
+      </c>
+      <c r="B35" t="n">
+        <v>31090637.89623569</v>
+      </c>
+      <c r="C35" t="n">
+        <v>4387244.906497965</v>
+      </c>
+      <c r="D35" t="n">
+        <v>23362895.97562808</v>
+      </c>
+      <c r="E35" t="n">
+        <v>0</v>
+      </c>
+      <c r="F35" t="n">
+        <v>54453533.87186377</v>
+      </c>
+      <c r="G35" t="n">
+        <v>4387244.906497965</v>
+      </c>
+      <c r="H35" t="n">
+        <v>2557523.584690922</v>
+      </c>
+      <c r="I35" t="n">
+        <v>-19626895.50306778</v>
+      </c>
+      <c r="J35" t="n">
+        <v>0</v>
+      </c>
+      <c r="K35" t="n">
+        <v>0</v>
+      </c>
+      <c r="L35" t="n">
+        <v>12779705.25101378</v>
+      </c>
+      <c r="M35" t="n">
+        <v>54551112.11099866</v>
+      </c>
+      <c r="N35" t="n">
+        <v>42603.78350836707</v>
+      </c>
+      <c r="O35" t="n">
+        <v>0</v>
+      </c>
+      <c r="P35" t="n">
+        <v>42603.78350836707</v>
+      </c>
+      <c r="Q35" t="n">
+        <v>42599.01750337926</v>
+      </c>
+      <c r="R35" t="n">
+        <v>0</v>
+      </c>
+      <c r="S35" t="n">
+        <v>0</v>
+      </c>
+      <c r="T35" t="n">
+        <v>0</v>
+      </c>
+      <c r="U35" t="n">
+        <v>4.766004987808616</v>
+      </c>
+      <c r="V35" t="n">
+        <v>3.273999929428101</v>
+      </c>
+      <c r="W35" t="n">
+        <v>54551112.11099866</v>
+      </c>
+      <c r="X35" t="n">
+        <v>54551112.11099866</v>
+      </c>
+      <c r="Y35" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z35" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA35" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB35" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC35" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD35" t="inlineStr">
+        <is>
+          <t>el_price_100_costs</t>
+        </is>
+      </c>
+      <c r="AE35" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_WtE\raw_results\CaL\20260203181524_el_price_100_costs</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>49637638.00808052</v>
+      </c>
+      <c r="B36" t="n">
+        <v>31289233.83448502</v>
+      </c>
+      <c r="C36" t="n">
+        <v>4406115.828823382</v>
+      </c>
+      <c r="D36" t="n">
+        <v>23501390.40939506</v>
+      </c>
+      <c r="E36" t="n">
+        <v>0</v>
+      </c>
+      <c r="F36" t="n">
+        <v>54790624.24388008</v>
+      </c>
+      <c r="G36" t="n">
+        <v>4406115.828823382</v>
+      </c>
+      <c r="H36" t="n">
+        <v>2573017.655303521</v>
+      </c>
+      <c r="I36" t="n">
+        <v>-24602063.2855968</v>
+      </c>
+      <c r="J36" t="n">
+        <v>0</v>
+      </c>
+      <c r="K36" t="n">
+        <v>0</v>
+      </c>
+      <c r="L36" t="n">
+        <v>12469943.56567033</v>
+      </c>
+      <c r="M36" t="n">
+        <v>49637638.00808052</v>
+      </c>
+      <c r="N36" t="n">
+        <v>41571.27343253568</v>
+      </c>
+      <c r="O36" t="n">
+        <v>0</v>
+      </c>
+      <c r="P36" t="n">
+        <v>41571.27343253568</v>
+      </c>
+      <c r="Q36" t="n">
+        <v>41566.47855223444</v>
+      </c>
+      <c r="R36" t="n">
+        <v>0</v>
+      </c>
+      <c r="S36" t="n">
+        <v>0</v>
+      </c>
+      <c r="T36" t="n">
+        <v>0</v>
+      </c>
+      <c r="U36" t="n">
+        <v>4.794880301223074</v>
+      </c>
+      <c r="V36" t="n">
+        <v>3.546999931335449</v>
+      </c>
+      <c r="W36" t="n">
+        <v>49637638.00808052</v>
+      </c>
+      <c r="X36" t="n">
+        <v>49637638.00808052</v>
+      </c>
+      <c r="Y36" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z36" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA36" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB36" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC36" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD36" t="inlineStr">
+        <is>
+          <t>el_price_125_costs</t>
+        </is>
+      </c>
+      <c r="AE36" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_WtE\raw_results\CaL\20260203181746_el_price_125_costs</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>44708664.97812186</v>
+      </c>
+      <c r="B37" t="n">
+        <v>31479609.3409155</v>
+      </c>
+      <c r="C37" t="n">
+        <v>4424205.631798112</v>
+      </c>
+      <c r="D37" t="n">
+        <v>23633332.99817676</v>
+      </c>
+      <c r="E37" t="n">
+        <v>0</v>
+      </c>
+      <c r="F37" t="n">
+        <v>55112942.33909227</v>
+      </c>
+      <c r="G37" t="n">
+        <v>4424205.631798112</v>
+      </c>
+      <c r="H37" t="n">
+        <v>2598877.293728911</v>
+      </c>
+      <c r="I37" t="n">
+        <v>-29628363.36563013</v>
+      </c>
+      <c r="J37" t="n">
+        <v>0</v>
+      </c>
+      <c r="K37" t="n">
+        <v>0</v>
+      </c>
+      <c r="L37" t="n">
+        <v>12201003.07913271</v>
+      </c>
+      <c r="M37" t="n">
+        <v>44708664.97812186</v>
+      </c>
+      <c r="N37" t="n">
+        <v>40674.83171475254</v>
+      </c>
+      <c r="O37" t="n">
+        <v>0</v>
+      </c>
+      <c r="P37" t="n">
+        <v>40674.83171475254</v>
+      </c>
+      <c r="Q37" t="n">
+        <v>40670.01026377569</v>
+      </c>
+      <c r="R37" t="n">
+        <v>0</v>
+      </c>
+      <c r="S37" t="n">
+        <v>0</v>
+      </c>
+      <c r="T37" t="n">
+        <v>0</v>
+      </c>
+      <c r="U37" t="n">
+        <v>4.82145097683823</v>
+      </c>
+      <c r="V37" t="n">
+        <v>3.086000204086304</v>
+      </c>
+      <c r="W37" t="n">
+        <v>44708664.97812186</v>
+      </c>
+      <c r="X37" t="n">
+        <v>44708664.97812186</v>
+      </c>
+      <c r="Y37" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z37" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA37" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC37" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD37" t="inlineStr">
+        <is>
+          <t>el_price_150_costs</t>
+        </is>
+      </c>
+      <c r="AE37" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_WtE\raw_results\CaL\20260203182014_el_price_150_costs</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>39763317.70086691</v>
+      </c>
+      <c r="B38" t="n">
+        <v>31644675.4328307</v>
+      </c>
+      <c r="C38" t="n">
+        <v>4439890.491350382</v>
+      </c>
+      <c r="D38" t="n">
+        <v>23747074.321913</v>
+      </c>
+      <c r="E38" t="n">
+        <v>0</v>
+      </c>
+      <c r="F38" t="n">
+        <v>55391749.75474371</v>
+      </c>
+      <c r="G38" t="n">
+        <v>4439890.491350382</v>
+      </c>
+      <c r="H38" t="n">
+        <v>2622589.083656741</v>
+      </c>
+      <c r="I38" t="n">
+        <v>-34670775.568021</v>
+      </c>
+      <c r="J38" t="n">
+        <v>0</v>
+      </c>
+      <c r="K38" t="n">
+        <v>0</v>
+      </c>
+      <c r="L38" t="n">
+        <v>11979863.93913708</v>
+      </c>
+      <c r="M38" t="n">
+        <v>39763317.70086691</v>
+      </c>
+      <c r="N38" t="n">
+        <v>39937.72339224516</v>
+      </c>
+      <c r="O38" t="n">
+        <v>0</v>
+      </c>
+      <c r="P38" t="n">
+        <v>39937.72339224516</v>
+      </c>
+      <c r="Q38" t="n">
+        <v>39932.87979712251</v>
+      </c>
+      <c r="R38" t="n">
+        <v>0</v>
+      </c>
+      <c r="S38" t="n">
+        <v>0</v>
+      </c>
+      <c r="T38" t="n">
+        <v>0</v>
+      </c>
+      <c r="U38" t="n">
+        <v>4.843595121557295</v>
+      </c>
+      <c r="V38" t="n">
+        <v>3.135999917984009</v>
+      </c>
+      <c r="W38" t="n">
+        <v>39763317.70086691</v>
+      </c>
+      <c r="X38" t="n">
+        <v>39763317.70086691</v>
+      </c>
+      <c r="Y38" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z38" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA38" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB38" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC38" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD38" t="inlineStr">
+        <is>
+          <t>el_price_175_costs</t>
+        </is>
+      </c>
+      <c r="AE38" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_WtE\raw_results\CaL\20260203182230_el_price_175_costs</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>34802702.85566229</v>
+      </c>
+      <c r="B39" t="n">
+        <v>31770005.71753078</v>
+      </c>
+      <c r="C39" t="n">
+        <v>4451799.587218337</v>
+      </c>
+      <c r="D39" t="n">
+        <v>23832960.21389318</v>
+      </c>
+      <c r="E39" t="n">
+        <v>0</v>
+      </c>
+      <c r="F39" t="n">
+        <v>55602965.93142396</v>
+      </c>
+      <c r="G39" t="n">
+        <v>4451799.587218337</v>
+      </c>
+      <c r="H39" t="n">
+        <v>2656059.808211191</v>
+      </c>
+      <c r="I39" t="n">
+        <v>-39748919.55638661</v>
+      </c>
+      <c r="J39" t="n">
+        <v>0</v>
+      </c>
+      <c r="K39" t="n">
+        <v>0</v>
+      </c>
+      <c r="L39" t="n">
+        <v>11840797.08519541</v>
+      </c>
+      <c r="M39" t="n">
+        <v>34802702.85566229</v>
+      </c>
+      <c r="N39" t="n">
+        <v>39474.18338279358</v>
+      </c>
+      <c r="O39" t="n">
+        <v>0</v>
+      </c>
+      <c r="P39" t="n">
+        <v>39474.18338279358</v>
+      </c>
+      <c r="Q39" t="n">
+        <v>39469.32361731802</v>
+      </c>
+      <c r="R39" t="n">
+        <v>0</v>
+      </c>
+      <c r="S39" t="n">
+        <v>0</v>
+      </c>
+      <c r="T39" t="n">
+        <v>0</v>
+      </c>
+      <c r="U39" t="n">
+        <v>4.859765475555238</v>
+      </c>
+      <c r="V39" t="n">
+        <v>3.036999940872192</v>
+      </c>
+      <c r="W39" t="n">
+        <v>34802702.85566229</v>
+      </c>
+      <c r="X39" t="n">
+        <v>34802702.85566229</v>
+      </c>
+      <c r="Y39" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z39" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA39" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB39" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC39" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD39" t="inlineStr">
+        <is>
+          <t>el_price_200_costs</t>
+        </is>
+      </c>
+      <c r="AE39" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_WtE\raw_results\CaL\20260203182449_el_price_200_costs</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
results cal (tax at 300) with higher el_price range
</commit_message>
<xml_diff>
--- a/dataCaseStudy_WtE/raw_results/CaL/Summary.xlsx
+++ b/dataCaseStudy_WtE/raw_results/CaL/Summary.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE39"/>
+  <dimension ref="A1:AE47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4496,6 +4496,830 @@
       <c r="AE39" t="inlineStr">
         <is>
           <t>dataCaseStudy_WtE\raw_results\CaL\20260203182449_el_price_200_costs</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>60347594.14647383</v>
+      </c>
+      <c r="B40" t="n">
+        <v>0</v>
+      </c>
+      <c r="C40" t="n">
+        <v>0</v>
+      </c>
+      <c r="D40" t="n">
+        <v>1800000</v>
+      </c>
+      <c r="E40" t="n">
+        <v>0</v>
+      </c>
+      <c r="F40" t="n">
+        <v>1800000</v>
+      </c>
+      <c r="G40" t="n">
+        <v>0</v>
+      </c>
+      <c r="H40" t="n">
+        <v>155.0546472912404</v>
+      </c>
+      <c r="I40" t="n">
+        <v>-5359875.275964417</v>
+      </c>
+      <c r="J40" t="n">
+        <v>0</v>
+      </c>
+      <c r="K40" t="n">
+        <v>0</v>
+      </c>
+      <c r="L40" t="n">
+        <v>63907314.36779096</v>
+      </c>
+      <c r="M40" t="n">
+        <v>60347594.14647383</v>
+      </c>
+      <c r="N40" t="n">
+        <v>213024.3812259698</v>
+      </c>
+      <c r="O40" t="n">
+        <v>0</v>
+      </c>
+      <c r="P40" t="n">
+        <v>213024.3812259698</v>
+      </c>
+      <c r="Q40" t="n">
+        <v>213024.3812259698</v>
+      </c>
+      <c r="R40" t="n">
+        <v>0</v>
+      </c>
+      <c r="S40" t="n">
+        <v>0</v>
+      </c>
+      <c r="T40" t="n">
+        <v>0</v>
+      </c>
+      <c r="U40" t="n">
+        <v>0</v>
+      </c>
+      <c r="V40" t="n">
+        <v>3.721000194549561</v>
+      </c>
+      <c r="W40" t="n">
+        <v>60347594.14647383</v>
+      </c>
+      <c r="X40" t="n">
+        <v>60347594.14647383</v>
+      </c>
+      <c r="Y40" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z40" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA40" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB40" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC40" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD40" t="inlineStr">
+        <is>
+          <t>el_price_50_costs</t>
+        </is>
+      </c>
+      <c r="AE40" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_WtE\raw_results\CaL\20260210170638_el_price_50_costs</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>54851112.11099866</v>
+      </c>
+      <c r="B41" t="n">
+        <v>31090637.89623569</v>
+      </c>
+      <c r="C41" t="n">
+        <v>4387244.906497965</v>
+      </c>
+      <c r="D41" t="n">
+        <v>23662895.97562808</v>
+      </c>
+      <c r="E41" t="n">
+        <v>0</v>
+      </c>
+      <c r="F41" t="n">
+        <v>54753533.87186377</v>
+      </c>
+      <c r="G41" t="n">
+        <v>4387244.906497965</v>
+      </c>
+      <c r="H41" t="n">
+        <v>2557523.584690922</v>
+      </c>
+      <c r="I41" t="n">
+        <v>-19626895.50306778</v>
+      </c>
+      <c r="J41" t="n">
+        <v>0</v>
+      </c>
+      <c r="K41" t="n">
+        <v>0</v>
+      </c>
+      <c r="L41" t="n">
+        <v>12779705.25101378</v>
+      </c>
+      <c r="M41" t="n">
+        <v>54851112.11099866</v>
+      </c>
+      <c r="N41" t="n">
+        <v>42603.78350836707</v>
+      </c>
+      <c r="O41" t="n">
+        <v>0</v>
+      </c>
+      <c r="P41" t="n">
+        <v>42603.78350836707</v>
+      </c>
+      <c r="Q41" t="n">
+        <v>42599.01750337926</v>
+      </c>
+      <c r="R41" t="n">
+        <v>0</v>
+      </c>
+      <c r="S41" t="n">
+        <v>0</v>
+      </c>
+      <c r="T41" t="n">
+        <v>0</v>
+      </c>
+      <c r="U41" t="n">
+        <v>4.766004987808616</v>
+      </c>
+      <c r="V41" t="n">
+        <v>2.91700005531311</v>
+      </c>
+      <c r="W41" t="n">
+        <v>54851112.11099866</v>
+      </c>
+      <c r="X41" t="n">
+        <v>54851112.11099866</v>
+      </c>
+      <c r="Y41" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z41" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA41" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB41" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC41" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD41" t="inlineStr">
+        <is>
+          <t>el_price_100_costs</t>
+        </is>
+      </c>
+      <c r="AE41" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_WtE\raw_results\CaL\20260210170855_el_price_100_costs</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>45008664.97812186</v>
+      </c>
+      <c r="B42" t="n">
+        <v>31479609.3409155</v>
+      </c>
+      <c r="C42" t="n">
+        <v>4424205.631798112</v>
+      </c>
+      <c r="D42" t="n">
+        <v>23933332.99817676</v>
+      </c>
+      <c r="E42" t="n">
+        <v>0</v>
+      </c>
+      <c r="F42" t="n">
+        <v>55412942.33909227</v>
+      </c>
+      <c r="G42" t="n">
+        <v>4424205.631798112</v>
+      </c>
+      <c r="H42" t="n">
+        <v>2598877.293728911</v>
+      </c>
+      <c r="I42" t="n">
+        <v>-29628363.36563013</v>
+      </c>
+      <c r="J42" t="n">
+        <v>0</v>
+      </c>
+      <c r="K42" t="n">
+        <v>0</v>
+      </c>
+      <c r="L42" t="n">
+        <v>12201003.07913271</v>
+      </c>
+      <c r="M42" t="n">
+        <v>45008664.97812186</v>
+      </c>
+      <c r="N42" t="n">
+        <v>40674.83171475254</v>
+      </c>
+      <c r="O42" t="n">
+        <v>0</v>
+      </c>
+      <c r="P42" t="n">
+        <v>40674.83171475254</v>
+      </c>
+      <c r="Q42" t="n">
+        <v>40670.01026377569</v>
+      </c>
+      <c r="R42" t="n">
+        <v>0</v>
+      </c>
+      <c r="S42" t="n">
+        <v>0</v>
+      </c>
+      <c r="T42" t="n">
+        <v>0</v>
+      </c>
+      <c r="U42" t="n">
+        <v>4.82145097683823</v>
+      </c>
+      <c r="V42" t="n">
+        <v>2.920000076293945</v>
+      </c>
+      <c r="W42" t="n">
+        <v>45008664.97812186</v>
+      </c>
+      <c r="X42" t="n">
+        <v>45008664.97812186</v>
+      </c>
+      <c r="Y42" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z42" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA42" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB42" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC42" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD42" t="inlineStr">
+        <is>
+          <t>el_price_150_costs</t>
+        </is>
+      </c>
+      <c r="AE42" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_WtE\raw_results\CaL\20260210171117_el_price_150_costs</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>35102702.85566229</v>
+      </c>
+      <c r="B43" t="n">
+        <v>31770005.71753078</v>
+      </c>
+      <c r="C43" t="n">
+        <v>4451799.587218337</v>
+      </c>
+      <c r="D43" t="n">
+        <v>24132960.21389318</v>
+      </c>
+      <c r="E43" t="n">
+        <v>0</v>
+      </c>
+      <c r="F43" t="n">
+        <v>55902965.93142396</v>
+      </c>
+      <c r="G43" t="n">
+        <v>4451799.587218337</v>
+      </c>
+      <c r="H43" t="n">
+        <v>2656059.808211191</v>
+      </c>
+      <c r="I43" t="n">
+        <v>-39748919.55638661</v>
+      </c>
+      <c r="J43" t="n">
+        <v>0</v>
+      </c>
+      <c r="K43" t="n">
+        <v>0</v>
+      </c>
+      <c r="L43" t="n">
+        <v>11840797.08519541</v>
+      </c>
+      <c r="M43" t="n">
+        <v>35102702.85566229</v>
+      </c>
+      <c r="N43" t="n">
+        <v>39474.18338279358</v>
+      </c>
+      <c r="O43" t="n">
+        <v>0</v>
+      </c>
+      <c r="P43" t="n">
+        <v>39474.18338279358</v>
+      </c>
+      <c r="Q43" t="n">
+        <v>39469.32361731802</v>
+      </c>
+      <c r="R43" t="n">
+        <v>0</v>
+      </c>
+      <c r="S43" t="n">
+        <v>0</v>
+      </c>
+      <c r="T43" t="n">
+        <v>0</v>
+      </c>
+      <c r="U43" t="n">
+        <v>4.859765475555238</v>
+      </c>
+      <c r="V43" t="n">
+        <v>2.898999929428101</v>
+      </c>
+      <c r="W43" t="n">
+        <v>35102702.85566229</v>
+      </c>
+      <c r="X43" t="n">
+        <v>35102702.85566229</v>
+      </c>
+      <c r="Y43" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z43" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA43" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB43" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC43" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD43" t="inlineStr">
+        <is>
+          <t>el_price_200_costs</t>
+        </is>
+      </c>
+      <c r="AE43" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_WtE\raw_results\CaL\20260210171340_el_price_200_costs</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>25096357.3266988</v>
+      </c>
+      <c r="B44" t="n">
+        <v>31990125.08539689</v>
+      </c>
+      <c r="C44" t="n">
+        <v>4472715.702270532</v>
+      </c>
+      <c r="D44" t="n">
+        <v>24282702.70480622</v>
+      </c>
+      <c r="E44" t="n">
+        <v>0</v>
+      </c>
+      <c r="F44" t="n">
+        <v>56272827.79020311</v>
+      </c>
+      <c r="G44" t="n">
+        <v>4472715.702270532</v>
+      </c>
+      <c r="H44" t="n">
+        <v>2888263.127648563</v>
+      </c>
+      <c r="I44" t="n">
+        <v>-50391711.21764924</v>
+      </c>
+      <c r="J44" t="n">
+        <v>0</v>
+      </c>
+      <c r="K44" t="n">
+        <v>0</v>
+      </c>
+      <c r="L44" t="n">
+        <v>11854261.92422584</v>
+      </c>
+      <c r="M44" t="n">
+        <v>25096357.3266988</v>
+      </c>
+      <c r="N44" t="n">
+        <v>39519.09308989099</v>
+      </c>
+      <c r="O44" t="n">
+        <v>0</v>
+      </c>
+      <c r="P44" t="n">
+        <v>39519.09308989099</v>
+      </c>
+      <c r="Q44" t="n">
+        <v>39514.20641408613</v>
+      </c>
+      <c r="R44" t="n">
+        <v>0</v>
+      </c>
+      <c r="S44" t="n">
+        <v>0</v>
+      </c>
+      <c r="T44" t="n">
+        <v>0</v>
+      </c>
+      <c r="U44" t="n">
+        <v>4.886675804847467</v>
+      </c>
+      <c r="V44" t="n">
+        <v>2.726000070571899</v>
+      </c>
+      <c r="W44" t="n">
+        <v>25096357.3266988</v>
+      </c>
+      <c r="X44" t="n">
+        <v>25096357.3266988</v>
+      </c>
+      <c r="Y44" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z44" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA44" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB44" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC44" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD44" t="inlineStr">
+        <is>
+          <t>el_price_250_costs</t>
+        </is>
+      </c>
+      <c r="AE44" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_WtE\raw_results\CaL\20260210171554_el_price_250_costs</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>14935899.7086328</v>
+      </c>
+      <c r="B45" t="n">
+        <v>32161570.19828518</v>
+      </c>
+      <c r="C45" t="n">
+        <v>4489006.707196956</v>
+      </c>
+      <c r="D45" t="n">
+        <v>24398244.72483689</v>
+      </c>
+      <c r="E45" t="n">
+        <v>0</v>
+      </c>
+      <c r="F45" t="n">
+        <v>56559814.92312206</v>
+      </c>
+      <c r="G45" t="n">
+        <v>4489006.707196956</v>
+      </c>
+      <c r="H45" t="n">
+        <v>3262983.45020072</v>
+      </c>
+      <c r="I45" t="n">
+        <v>-61526550.34251533</v>
+      </c>
+      <c r="J45" t="n">
+        <v>0</v>
+      </c>
+      <c r="K45" t="n">
+        <v>0</v>
+      </c>
+      <c r="L45" t="n">
+        <v>12150644.97062838</v>
+      </c>
+      <c r="M45" t="n">
+        <v>14935899.7086328</v>
+      </c>
+      <c r="N45" t="n">
+        <v>40507.05606360164</v>
+      </c>
+      <c r="O45" t="n">
+        <v>0</v>
+      </c>
+      <c r="P45" t="n">
+        <v>40507.05606360164</v>
+      </c>
+      <c r="Q45" t="n">
+        <v>40502.14990209352</v>
+      </c>
+      <c r="R45" t="n">
+        <v>0</v>
+      </c>
+      <c r="S45" t="n">
+        <v>0</v>
+      </c>
+      <c r="T45" t="n">
+        <v>0</v>
+      </c>
+      <c r="U45" t="n">
+        <v>4.906161507022792</v>
+      </c>
+      <c r="V45" t="n">
+        <v>2.763000011444092</v>
+      </c>
+      <c r="W45" t="n">
+        <v>14935899.7086328</v>
+      </c>
+      <c r="X45" t="n">
+        <v>14935899.7086328</v>
+      </c>
+      <c r="Y45" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z45" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA45" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC45" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD45" t="inlineStr">
+        <is>
+          <t>el_price_300_costs</t>
+        </is>
+      </c>
+      <c r="AE45" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_WtE\raw_results\CaL\20260210171812_el_price_300_costs</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>4580393.309028087</v>
+      </c>
+      <c r="B46" t="n">
+        <v>32328899.56987783</v>
+      </c>
+      <c r="C46" t="n">
+        <v>4504906.62741648</v>
+      </c>
+      <c r="D46" t="n">
+        <v>24510104.1827603</v>
+      </c>
+      <c r="E46" t="n">
+        <v>0</v>
+      </c>
+      <c r="F46" t="n">
+        <v>56839003.75263813</v>
+      </c>
+      <c r="G46" t="n">
+        <v>4504906.62741648</v>
+      </c>
+      <c r="H46" t="n">
+        <v>3765495.501193692</v>
+      </c>
+      <c r="I46" t="n">
+        <v>-73172838.22538382</v>
+      </c>
+      <c r="J46" t="n">
+        <v>0</v>
+      </c>
+      <c r="K46" t="n">
+        <v>0</v>
+      </c>
+      <c r="L46" t="n">
+        <v>12643825.6531636</v>
+      </c>
+      <c r="M46" t="n">
+        <v>4580393.309028087</v>
+      </c>
+      <c r="N46" t="n">
+        <v>42151.00945914153</v>
+      </c>
+      <c r="O46" t="n">
+        <v>0</v>
+      </c>
+      <c r="P46" t="n">
+        <v>42151.00945914153</v>
+      </c>
+      <c r="Q46" t="n">
+        <v>42146.08551054534</v>
+      </c>
+      <c r="R46" t="n">
+        <v>0</v>
+      </c>
+      <c r="S46" t="n">
+        <v>0</v>
+      </c>
+      <c r="T46" t="n">
+        <v>0</v>
+      </c>
+      <c r="U46" t="n">
+        <v>4.923948596172322</v>
+      </c>
+      <c r="V46" t="n">
+        <v>2.730000019073486</v>
+      </c>
+      <c r="W46" t="n">
+        <v>4580393.309028087</v>
+      </c>
+      <c r="X46" t="n">
+        <v>4580393.309028087</v>
+      </c>
+      <c r="Y46" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z46" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA46" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB46" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC46" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD46" t="inlineStr">
+        <is>
+          <t>el_price_350_costs</t>
+        </is>
+      </c>
+      <c r="AE46" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_WtE\raw_results\CaL\20260210172034_el_price_350_costs</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>-5963256.334402483</v>
+      </c>
+      <c r="B47" t="n">
+        <v>32492712.19741435</v>
+      </c>
+      <c r="C47" t="n">
+        <v>4520472.380661057</v>
+      </c>
+      <c r="D47" t="n">
+        <v>24618820.51788848</v>
+      </c>
+      <c r="E47" t="n">
+        <v>0</v>
+      </c>
+      <c r="F47" t="n">
+        <v>57111532.71530282</v>
+      </c>
+      <c r="G47" t="n">
+        <v>4520472.380661057</v>
+      </c>
+      <c r="H47" t="n">
+        <v>4239155.782364045</v>
+      </c>
+      <c r="I47" t="n">
+        <v>-84947988.12293488</v>
+      </c>
+      <c r="J47" t="n">
+        <v>0</v>
+      </c>
+      <c r="K47" t="n">
+        <v>0</v>
+      </c>
+      <c r="L47" t="n">
+        <v>13113570.91020447</v>
+      </c>
+      <c r="M47" t="n">
+        <v>-5963256.334402483</v>
+      </c>
+      <c r="N47" t="n">
+        <v>43716.84332302142</v>
+      </c>
+      <c r="O47" t="n">
+        <v>0</v>
+      </c>
+      <c r="P47" t="n">
+        <v>43716.84332302142</v>
+      </c>
+      <c r="Q47" t="n">
+        <v>43711.90303401487</v>
+      </c>
+      <c r="R47" t="n">
+        <v>0</v>
+      </c>
+      <c r="S47" t="n">
+        <v>0</v>
+      </c>
+      <c r="T47" t="n">
+        <v>0</v>
+      </c>
+      <c r="U47" t="n">
+        <v>4.940289006514293</v>
+      </c>
+      <c r="V47" t="n">
+        <v>2.747999906539917</v>
+      </c>
+      <c r="W47" t="n">
+        <v>-5963256.334402483</v>
+      </c>
+      <c r="X47" t="n">
+        <v>-5963256.334402483</v>
+      </c>
+      <c r="Y47" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z47" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA47" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB47" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC47" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD47" t="inlineStr">
+        <is>
+          <t>el_price_400_costs</t>
+        </is>
+      </c>
+      <c r="AE47" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_WtE\raw_results\CaL\20260210172303_el_price_400_costs</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
results mea and mea timeless
</commit_message>
<xml_diff>
--- a/dataCaseStudy_WtE/raw_results/CaL/Summary.xlsx
+++ b/dataCaseStudy_WtE/raw_results/CaL/Summary.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE59"/>
+  <dimension ref="A1:AE60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6556,6 +6556,109 @@
       <c r="AE59" t="inlineStr">
         <is>
           <t>dataCaseStudy_WtE\raw_results\CaL\20260409190648_el_price_400_costs</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="n">
+        <v>51528530.84522993</v>
+      </c>
+      <c r="B60" t="n">
+        <v>31090637.89623569</v>
+      </c>
+      <c r="C60" t="n">
+        <v>4387244.906497963</v>
+      </c>
+      <c r="D60" t="n">
+        <v>23662895.97562808</v>
+      </c>
+      <c r="E60" t="n">
+        <v>0</v>
+      </c>
+      <c r="F60" t="n">
+        <v>54753533.87186377</v>
+      </c>
+      <c r="G60" t="n">
+        <v>4387244.906497963</v>
+      </c>
+      <c r="H60" t="n">
+        <v>2557368.530043631</v>
+      </c>
+      <c r="I60" t="n">
+        <v>-22949106.57586608</v>
+      </c>
+      <c r="J60" t="n">
+        <v>0</v>
+      </c>
+      <c r="K60" t="n">
+        <v>0</v>
+      </c>
+      <c r="L60" t="n">
+        <v>12779490.11269065</v>
+      </c>
+      <c r="M60" t="n">
+        <v>51528530.84522993</v>
+      </c>
+      <c r="N60" t="n">
+        <v>42603.06638062331</v>
+      </c>
+      <c r="O60" t="n">
+        <v>0</v>
+      </c>
+      <c r="P60" t="n">
+        <v>42603.06638062331</v>
+      </c>
+      <c r="Q60" t="n">
+        <v>42598.3003756355</v>
+      </c>
+      <c r="R60" t="n">
+        <v>0</v>
+      </c>
+      <c r="S60" t="n">
+        <v>0</v>
+      </c>
+      <c r="T60" t="n">
+        <v>0</v>
+      </c>
+      <c r="U60" t="n">
+        <v>4.766004987808613</v>
+      </c>
+      <c r="V60" t="n">
+        <v>3.472999811172485</v>
+      </c>
+      <c r="W60" t="n">
+        <v>51528530.84522993</v>
+      </c>
+      <c r="X60" t="n">
+        <v>51528530.84522993</v>
+      </c>
+      <c r="Y60" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z60" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA60" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB60" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC60" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD60" t="inlineStr">
+        <is>
+          <t>el_price_100_costs</t>
+        </is>
+      </c>
+      <c r="AE60" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_WtE\raw_results\CaL\20260410164847_el_price_100_costs</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
results wte with opex var mea
</commit_message>
<xml_diff>
--- a/dataCaseStudy_WtE/raw_results/CaL/Summary.xlsx
+++ b/dataCaseStudy_WtE/raw_results/CaL/Summary.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE74"/>
+  <dimension ref="A1:AE79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8101,6 +8101,521 @@
       <c r="AE74" t="inlineStr">
         <is>
           <t>dataCaseStudy_WtE\raw_results\CaL\20260417161345_el_price_300_costs</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="n">
+        <v>51058685.68229314</v>
+      </c>
+      <c r="B75" t="n">
+        <v>30787735.34465664</v>
+      </c>
+      <c r="C75" t="n">
+        <v>4388356.629693229</v>
+      </c>
+      <c r="D75" t="n">
+        <v>23483931.62107569</v>
+      </c>
+      <c r="E75" t="n">
+        <v>0</v>
+      </c>
+      <c r="F75" t="n">
+        <v>54271666.96573234</v>
+      </c>
+      <c r="G75" t="n">
+        <v>4388356.629693229</v>
+      </c>
+      <c r="H75" t="n">
+        <v>2557187.18601264</v>
+      </c>
+      <c r="I75" t="n">
+        <v>-22941640.69115957</v>
+      </c>
+      <c r="J75" t="n">
+        <v>0</v>
+      </c>
+      <c r="K75" t="n">
+        <v>0</v>
+      </c>
+      <c r="L75" t="n">
+        <v>12783115.5920145</v>
+      </c>
+      <c r="M75" t="n">
+        <v>51058685.68229314</v>
+      </c>
+      <c r="N75" t="n">
+        <v>42615.15097374347</v>
+      </c>
+      <c r="O75" t="n">
+        <v>0</v>
+      </c>
+      <c r="P75" t="n">
+        <v>42615.15097374347</v>
+      </c>
+      <c r="Q75" t="n">
+        <v>42610.38530671498</v>
+      </c>
+      <c r="R75" t="n">
+        <v>0</v>
+      </c>
+      <c r="S75" t="n">
+        <v>0</v>
+      </c>
+      <c r="T75" t="n">
+        <v>0</v>
+      </c>
+      <c r="U75" t="n">
+        <v>4.765667028478242</v>
+      </c>
+      <c r="V75" t="n">
+        <v>4.059000015258789</v>
+      </c>
+      <c r="W75" t="n">
+        <v>51058685.68229314</v>
+      </c>
+      <c r="X75" t="n">
+        <v>51058685.68229314</v>
+      </c>
+      <c r="Y75" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z75" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA75" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB75" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC75" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD75" t="inlineStr">
+        <is>
+          <t>el_price_100_costs</t>
+        </is>
+      </c>
+      <c r="AE75" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_WtE\raw_results\CaL\20260425224429_el_price_100_costs</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="n">
+        <v>39558643.1936384</v>
+      </c>
+      <c r="B76" t="n">
+        <v>31175531.31469489</v>
+      </c>
+      <c r="C76" t="n">
+        <v>4425678.503486734</v>
+      </c>
+      <c r="D76" t="n">
+        <v>23753599.06207174</v>
+      </c>
+      <c r="E76" t="n">
+        <v>0</v>
+      </c>
+      <c r="F76" t="n">
+        <v>54929130.37676664</v>
+      </c>
+      <c r="G76" t="n">
+        <v>4425678.503486734</v>
+      </c>
+      <c r="H76" t="n">
+        <v>2598499.60273234</v>
+      </c>
+      <c r="I76" t="n">
+        <v>-34600202.85552283</v>
+      </c>
+      <c r="J76" t="n">
+        <v>0</v>
+      </c>
+      <c r="K76" t="n">
+        <v>0</v>
+      </c>
+      <c r="L76" t="n">
+        <v>12205537.56617552</v>
+      </c>
+      <c r="M76" t="n">
+        <v>39558643.1936384</v>
+      </c>
+      <c r="N76" t="n">
+        <v>40689.94623061863</v>
+      </c>
+      <c r="O76" t="n">
+        <v>0</v>
+      </c>
+      <c r="P76" t="n">
+        <v>40689.94623061863</v>
+      </c>
+      <c r="Q76" t="n">
+        <v>40685.12522058505</v>
+      </c>
+      <c r="R76" t="n">
+        <v>0</v>
+      </c>
+      <c r="S76" t="n">
+        <v>0</v>
+      </c>
+      <c r="T76" t="n">
+        <v>0</v>
+      </c>
+      <c r="U76" t="n">
+        <v>4.821010033581917</v>
+      </c>
+      <c r="V76" t="n">
+        <v>3.353000164031982</v>
+      </c>
+      <c r="W76" t="n">
+        <v>39558643.1936384</v>
+      </c>
+      <c r="X76" t="n">
+        <v>39558643.1936384</v>
+      </c>
+      <c r="Y76" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z76" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA76" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB76" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC76" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD76" t="inlineStr">
+        <is>
+          <t>el_price_150_costs</t>
+        </is>
+      </c>
+      <c r="AE76" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_WtE\raw_results\CaL\20260425224701_el_price_150_costs</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="n">
+        <v>27997561.75950783</v>
+      </c>
+      <c r="B77" t="n">
+        <v>31449528.01604342</v>
+      </c>
+      <c r="C77" t="n">
+        <v>4452048.221322012</v>
+      </c>
+      <c r="D77" t="n">
+        <v>23941917.38006485</v>
+      </c>
+      <c r="E77" t="n">
+        <v>0</v>
+      </c>
+      <c r="F77" t="n">
+        <v>55391445.39610826</v>
+      </c>
+      <c r="G77" t="n">
+        <v>4452048.221322012</v>
+      </c>
+      <c r="H77" t="n">
+        <v>2654330.786248672</v>
+      </c>
+      <c r="I77" t="n">
+        <v>-46369089.87749237</v>
+      </c>
+      <c r="J77" t="n">
+        <v>0</v>
+      </c>
+      <c r="K77" t="n">
+        <v>0</v>
+      </c>
+      <c r="L77" t="n">
+        <v>11868827.23332126</v>
+      </c>
+      <c r="M77" t="n">
+        <v>27997561.75950783</v>
+      </c>
+      <c r="N77" t="n">
+        <v>39567.61455742401</v>
+      </c>
+      <c r="O77" t="n">
+        <v>0</v>
+      </c>
+      <c r="P77" t="n">
+        <v>39567.61455742401</v>
+      </c>
+      <c r="Q77" t="n">
+        <v>39562.75744440419</v>
+      </c>
+      <c r="R77" t="n">
+        <v>0</v>
+      </c>
+      <c r="S77" t="n">
+        <v>0</v>
+      </c>
+      <c r="T77" t="n">
+        <v>0</v>
+      </c>
+      <c r="U77" t="n">
+        <v>4.857113019835499</v>
+      </c>
+      <c r="V77" t="n">
+        <v>3.33899998664856</v>
+      </c>
+      <c r="W77" t="n">
+        <v>27997561.75950783</v>
+      </c>
+      <c r="X77" t="n">
+        <v>27997561.75950783</v>
+      </c>
+      <c r="Y77" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z77" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA77" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB77" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC77" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD77" t="inlineStr">
+        <is>
+          <t>el_price_200_costs</t>
+        </is>
+      </c>
+      <c r="AE77" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_WtE\raw_results\CaL\20260425224922_el_price_200_costs</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="n">
+        <v>16338227.29707677</v>
+      </c>
+      <c r="B78" t="n">
+        <v>31652283.18563704</v>
+      </c>
+      <c r="C78" t="n">
+        <v>4471561.582561448</v>
+      </c>
+      <c r="D78" t="n">
+        <v>24079832.38165812</v>
+      </c>
+      <c r="E78" t="n">
+        <v>0</v>
+      </c>
+      <c r="F78" t="n">
+        <v>55732115.56729516</v>
+      </c>
+      <c r="G78" t="n">
+        <v>4471561.582561448</v>
+      </c>
+      <c r="H78" t="n">
+        <v>2884063.285821915</v>
+      </c>
+      <c r="I78" t="n">
+        <v>-58652963.22934026</v>
+      </c>
+      <c r="J78" t="n">
+        <v>0</v>
+      </c>
+      <c r="K78" t="n">
+        <v>0</v>
+      </c>
+      <c r="L78" t="n">
+        <v>11903450.09073851</v>
+      </c>
+      <c r="M78" t="n">
+        <v>16338227.29707677</v>
+      </c>
+      <c r="N78" t="n">
+        <v>39683.04884933559</v>
+      </c>
+      <c r="O78" t="n">
+        <v>0</v>
+      </c>
+      <c r="P78" t="n">
+        <v>39683.04884933559</v>
+      </c>
+      <c r="Q78" t="n">
+        <v>39678.16696912838</v>
+      </c>
+      <c r="R78" t="n">
+        <v>0</v>
+      </c>
+      <c r="S78" t="n">
+        <v>0</v>
+      </c>
+      <c r="T78" t="n">
+        <v>0</v>
+      </c>
+      <c r="U78" t="n">
+        <v>4.881880207205398</v>
+      </c>
+      <c r="V78" t="n">
+        <v>3.46399998664856</v>
+      </c>
+      <c r="W78" t="n">
+        <v>16338227.29707677</v>
+      </c>
+      <c r="X78" t="n">
+        <v>16338227.29707677</v>
+      </c>
+      <c r="Y78" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z78" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA78" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB78" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC78" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD78" t="inlineStr">
+        <is>
+          <t>el_price_250_costs</t>
+        </is>
+      </c>
+      <c r="AE78" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_WtE\raw_results\CaL\20260425225154_el_price_250_costs</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="n">
+        <v>4526518.000937495</v>
+      </c>
+      <c r="B79" t="n">
+        <v>31816843.96321993</v>
+      </c>
+      <c r="C79" t="n">
+        <v>4487399.077138051</v>
+      </c>
+      <c r="D79" t="n">
+        <v>24190741.61294693</v>
+      </c>
+      <c r="E79" t="n">
+        <v>0</v>
+      </c>
+      <c r="F79" t="n">
+        <v>56007585.57616685</v>
+      </c>
+      <c r="G79" t="n">
+        <v>4487399.077138051</v>
+      </c>
+      <c r="H79" t="n">
+        <v>3256171.542092193</v>
+      </c>
+      <c r="I79" t="n">
+        <v>-71429718.12543741</v>
+      </c>
+      <c r="J79" t="n">
+        <v>0</v>
+      </c>
+      <c r="K79" t="n">
+        <v>0</v>
+      </c>
+      <c r="L79" t="n">
+        <v>12205079.9309778</v>
+      </c>
+      <c r="M79" t="n">
+        <v>4526518.000937495</v>
+      </c>
+      <c r="N79" t="n">
+        <v>40688.50036256314</v>
+      </c>
+      <c r="O79" t="n">
+        <v>0</v>
+      </c>
+      <c r="P79" t="n">
+        <v>40688.50036256314</v>
+      </c>
+      <c r="Q79" t="n">
+        <v>40683.59976992603</v>
+      </c>
+      <c r="R79" t="n">
+        <v>0</v>
+      </c>
+      <c r="S79" t="n">
+        <v>0</v>
+      </c>
+      <c r="T79" t="n">
+        <v>0</v>
+      </c>
+      <c r="U79" t="n">
+        <v>4.900592637133351</v>
+      </c>
+      <c r="V79" t="n">
+        <v>3.264999866485596</v>
+      </c>
+      <c r="W79" t="n">
+        <v>4526518.000937495</v>
+      </c>
+      <c r="X79" t="n">
+        <v>4526518.000937495</v>
+      </c>
+      <c r="Y79" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z79" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA79" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB79" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC79" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD79" t="inlineStr">
+        <is>
+          <t>el_price_300_costs</t>
+        </is>
+      </c>
+      <c r="AE79" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_WtE\raw_results\CaL\20260425225441_el_price_300_costs</t>
         </is>
       </c>
     </row>

</xml_diff>